<commit_message>
add previous tip button
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93ECEF60-CDCB-4538-86F2-A7F2127B1623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D00EAD0-2659-4FFF-A44E-0EFE74D84F29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1900" yWindow="1900" windowWidth="31590" windowHeight="15280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2712" uniqueCount="2557">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2715" uniqueCount="2560">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -22138,6 +22138,17 @@
   </si>
   <si>
     <t>Draw all ranges except for weapons subject to elevation using ellipses</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>TipDialogPrevious</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Previous tip</t>
+  </si>
+  <si>
+    <t>上一提示</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -32512,6 +32523,17 @@
         <v>2556</v>
       </c>
     </row>
+    <row r="907" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A907" s="4" t="s">
+        <v>2557</v>
+      </c>
+      <c r="B907" s="5" t="s">
+        <v>2559</v>
+      </c>
+      <c r="C907" s="3" t="s">
+        <v>2558</v>
+      </c>
+    </row>
     <row r="910" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A910" s="7"/>
     </row>

</xml_diff>

<commit_message>
add translation for spotlight combobox
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E213F9B4-3A27-4782-BB93-B4F7DA5E228B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3ACBBD4-98DB-49D6-9496-EE427122F492}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1900" yWindow="1900" windowWidth="31590" windowHeight="15280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2721" uniqueCount="2566">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2730" uniqueCount="2575">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -22133,6 +22133,36 @@
   </si>
   <si>
     <t>重置工具栏</t>
+  </si>
+  <si>
+    <t>0 - No spotlight</t>
+  </si>
+  <si>
+    <t>1 - Rules.ini setting</t>
+  </si>
+  <si>
+    <t>2 - Circle / Direction</t>
+  </si>
+  <si>
+    <t>StructSpotlight.0</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>StructSpotlight.1</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>StructSpotlight.2</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>0 - 无聚光灯</t>
+  </si>
+  <si>
+    <t>1 - 使用Rules设置</t>
+  </si>
+  <si>
+    <t>2 - 圆/目标聚光灯</t>
   </si>
 </sst>
 </file>
@@ -22538,7 +22568,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C909"/>
+  <dimension ref="A1:C912"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="4" customWidth="1"/>
@@ -32528,6 +32558,39 @@
         <v>2559</v>
       </c>
     </row>
+    <row r="910" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A910" s="4" t="s">
+        <v>2569</v>
+      </c>
+      <c r="B910" s="5" t="s">
+        <v>2572</v>
+      </c>
+      <c r="C910" s="3" t="s">
+        <v>2566</v>
+      </c>
+    </row>
+    <row r="911" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A911" s="4" t="s">
+        <v>2570</v>
+      </c>
+      <c r="B911" s="5" t="s">
+        <v>2573</v>
+      </c>
+      <c r="C911" s="3" t="s">
+        <v>2567</v>
+      </c>
+    </row>
+    <row r="912" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A912" s="4" t="s">
+        <v>2571</v>
+      </c>
+      <c r="B912" s="5" t="s">
+        <v>2574</v>
+      </c>
+      <c r="C912" s="3" t="s">
+        <v>2568</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add Techno property brush
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3ACBBD4-98DB-49D6-9496-EE427122F492}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA9B63EB-11C7-48F9-8BF9-817C5EA2DFE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1900" yWindow="1900" windowWidth="31590" windowHeight="15280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2240" yWindow="2240" windowWidth="31590" windowHeight="15280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2730" uniqueCount="2575">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2736" uniqueCount="2579">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -22163,6 +22163,20 @@
   </si>
   <si>
     <t>2 - 圆/目标聚光灯</t>
+  </si>
+  <si>
+    <t>TechnoOptionsCaption</t>
+  </si>
+  <si>
+    <t>通用格式刷</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Techno Property Brush</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>PropertyBrushTechno</t>
   </si>
 </sst>
 </file>
@@ -22568,7 +22582,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C912"/>
+  <dimension ref="A1:C914"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="4" customWidth="1"/>
@@ -32591,6 +32605,28 @@
         <v>2568</v>
       </c>
     </row>
+    <row r="913" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A913" s="4" t="s">
+        <v>2575</v>
+      </c>
+      <c r="B913" s="5" t="s">
+        <v>2576</v>
+      </c>
+      <c r="C913" s="3" t="s">
+        <v>2577</v>
+      </c>
+    </row>
+    <row r="914" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A914" s="4" t="s">
+        <v>2578</v>
+      </c>
+      <c r="B914" s="5" t="s">
+        <v>2576</v>
+      </c>
+      <c r="C914" s="3" t="s">
+        <v>2577</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add new option to show bridge overlay
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA9B63EB-11C7-48F9-8BF9-817C5EA2DFE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{543A9372-2DA2-478E-8EDA-A61F04A609F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2240" yWindow="2240" windowWidth="31590" windowHeight="15280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2736" uniqueCount="2579">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2739" uniqueCount="2582">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -22177,6 +22177,16 @@
   </si>
   <si>
     <t>PropertyBrushTechno</t>
+  </si>
+  <si>
+    <t>Options.DisplayBridgeOverlay</t>
+  </si>
+  <si>
+    <t>Display invisible bridge overlays in numbers</t>
+  </si>
+  <si>
+    <t>以数字显示不可见的桥梁覆盖物</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -22582,7 +22592,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C914"/>
+  <dimension ref="A1:C915"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="4" customWidth="1"/>
@@ -32627,6 +32637,17 @@
         <v>2577</v>
       </c>
     </row>
+    <row r="915" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A915" s="4" t="s">
+        <v>2579</v>
+      </c>
+      <c r="B915" s="5" t="s">
+        <v>2581</v>
+      </c>
+      <c r="C915" s="3" t="s">
+        <v>2580</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add disable auto connect wall
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{543A9372-2DA2-478E-8EDA-A61F04A609F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66C5F01F-8546-4655-9C79-19BF3263C3FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2240" yWindow="2240" windowWidth="31590" windowHeight="15280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2739" uniqueCount="2582">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2742" uniqueCount="2585">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -22186,6 +22186,17 @@
   </si>
   <si>
     <t>以数字显示不可见的桥梁覆盖物</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Disable Auto Connect Wall</t>
+  </si>
+  <si>
+    <t>Menu.Options.DisableAutoConnectWall</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>禁止自动连接围墙</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -22592,7 +22603,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C915"/>
+  <dimension ref="A1:C916"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="4" customWidth="1"/>
@@ -32648,6 +32659,17 @@
         <v>2580</v>
       </c>
     </row>
+    <row r="916" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A916" s="4" t="s">
+        <v>2583</v>
+      </c>
+      <c r="B916" s="5" t="s">
+        <v>2584</v>
+      </c>
+      <c r="C916" s="3" t="s">
+        <v>2582</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
support veinhole logic, rewrite overlay combobox loading
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A69430B-E5AA-469B-9BDF-BE3188D36056}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90139EE7-E951-4B92-92C1-BB771D05B9C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2240" yWindow="2240" windowWidth="31590" windowHeight="15280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2745" uniqueCount="2588">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2748" uniqueCount="2591">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -22207,6 +22207,16 @@
   </si>
   <si>
     <t>双击打开地图文件时，从地图目录加载资源文件</t>
+  </si>
+  <si>
+    <t>Enable veinhole logic</t>
+  </si>
+  <si>
+    <t>Options.EnableVeinholeLogic</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>启用泰伯利亚藤蔓（蔓孔）逻辑</t>
   </si>
 </sst>
 </file>
@@ -22612,7 +22622,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C917"/>
+  <dimension ref="A1:C918"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="4" customWidth="1"/>
@@ -32690,6 +32700,17 @@
         <v>2586</v>
       </c>
     </row>
+    <row r="918" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A918" s="4" t="s">
+        <v>2589</v>
+      </c>
+      <c r="B918" s="5" t="s">
+        <v>2590</v>
+      </c>
+      <c r="C918" s="3" t="s">
+        <v>2588</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
reduce unnecessary file loading checks
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90139EE7-E951-4B92-92C1-BB771D05B9C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80AA0536-FF3B-4C9E-88B6-8E7DE506D008}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2240" yWindow="2240" windowWidth="31590" windowHeight="15280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21378,9 +21378,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>Display remapble colors of overlays</t>
-  </si>
-  <si>
     <t>显示围墙覆盖物的所属色</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -22217,6 +22214,10 @@
   </si>
   <si>
     <t>启用泰伯利亚藤蔓（蔓孔）逻辑</t>
+  </si>
+  <si>
+    <t>Display remapable colors of overlays</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -30219,7 +30220,7 @@
         <v>701</v>
       </c>
       <c r="B692" s="5" t="s">
-        <v>2550</v>
+        <v>2549</v>
       </c>
       <c r="C692" s="3" t="s">
         <v>1100</v>
@@ -31803,183 +31804,183 @@
         <v>2355</v>
       </c>
       <c r="B836" s="5" t="s">
-        <v>2357</v>
+        <v>2356</v>
       </c>
       <c r="C836" s="3" t="s">
-        <v>2356</v>
+        <v>2590</v>
       </c>
     </row>
     <row r="837" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A837" s="4" t="s">
-        <v>2360</v>
+        <v>2359</v>
       </c>
       <c r="B837" s="5" t="s">
-        <v>2359</v>
+        <v>2358</v>
       </c>
       <c r="C837" s="3" t="s">
-        <v>2358</v>
+        <v>2357</v>
       </c>
     </row>
     <row r="838" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A838" s="4" t="s">
+        <v>2360</v>
+      </c>
+      <c r="B838" s="5" t="s">
         <v>2361</v>
       </c>
-      <c r="B838" s="5" t="s">
+      <c r="C838" s="3" t="s">
         <v>2362</v>
-      </c>
-      <c r="C838" s="3" t="s">
-        <v>2363</v>
       </c>
     </row>
     <row r="839" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A839" s="4" t="s">
+        <v>2363</v>
+      </c>
+      <c r="B839" s="5" t="s">
         <v>2364</v>
       </c>
-      <c r="B839" s="5" t="s">
+      <c r="C839" s="3" t="s">
         <v>2365</v>
-      </c>
-      <c r="C839" s="3" t="s">
-        <v>2366</v>
       </c>
     </row>
     <row r="840" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A840" s="4" t="s">
+        <v>2366</v>
+      </c>
+      <c r="B840" s="5" t="s">
         <v>2367</v>
       </c>
-      <c r="B840" s="5" t="s">
+      <c r="C840" s="3" t="s">
         <v>2368</v>
-      </c>
-      <c r="C840" s="3" t="s">
-        <v>2369</v>
       </c>
     </row>
     <row r="841" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A841" s="4" t="s">
+        <v>2369</v>
+      </c>
+      <c r="B841" s="5" t="s">
         <v>2370</v>
       </c>
-      <c r="B841" s="5" t="s">
+      <c r="C841" s="3" t="s">
         <v>2371</v>
-      </c>
-      <c r="C841" s="3" t="s">
-        <v>2372</v>
       </c>
     </row>
     <row r="842" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A842" s="4" t="s">
+        <v>2372</v>
+      </c>
+      <c r="B842" s="5" t="s">
         <v>2373</v>
       </c>
-      <c r="B842" s="5" t="s">
+      <c r="C842" s="3" t="s">
         <v>2374</v>
-      </c>
-      <c r="C842" s="3" t="s">
-        <v>2375</v>
       </c>
     </row>
     <row r="843" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A843" s="4" t="s">
+        <v>2375</v>
+      </c>
+      <c r="B843" s="5" t="s">
         <v>2376</v>
       </c>
-      <c r="B843" s="5" t="s">
-        <v>2377</v>
-      </c>
       <c r="C843" s="3" t="s">
-        <v>2366</v>
+        <v>2365</v>
       </c>
     </row>
     <row r="844" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A844" s="4" t="s">
+        <v>2377</v>
+      </c>
+      <c r="B844" s="5" t="s">
         <v>2378</v>
       </c>
-      <c r="B844" s="5" t="s">
+      <c r="C844" s="3" t="s">
         <v>2379</v>
-      </c>
-      <c r="C844" s="3" t="s">
-        <v>2380</v>
       </c>
     </row>
     <row r="845" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A845" s="4" t="s">
-        <v>2381</v>
+        <v>2380</v>
       </c>
       <c r="B845" s="5" t="s">
+        <v>2364</v>
+      </c>
+      <c r="C845" s="3" t="s">
         <v>2365</v>
-      </c>
-      <c r="C845" s="3" t="s">
-        <v>2366</v>
       </c>
     </row>
     <row r="846" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A846" s="4" t="s">
+        <v>2381</v>
+      </c>
+      <c r="B846" s="5" t="s">
         <v>2382</v>
       </c>
-      <c r="B846" s="5" t="s">
+      <c r="C846" s="3" t="s">
         <v>2383</v>
-      </c>
-      <c r="C846" s="3" t="s">
-        <v>2384</v>
       </c>
     </row>
     <row r="847" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A847" s="4" t="s">
+        <v>2384</v>
+      </c>
+      <c r="B847" s="5" t="s">
         <v>2385</v>
       </c>
-      <c r="B847" s="5" t="s">
-        <v>2386</v>
-      </c>
       <c r="C847" s="3" t="s">
-        <v>2372</v>
+        <v>2371</v>
       </c>
     </row>
     <row r="848" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A848" s="4" t="s">
+        <v>2386</v>
+      </c>
+      <c r="B848" s="5" t="s">
         <v>2387</v>
       </c>
-      <c r="B848" s="5" t="s">
+      <c r="C848" s="3" t="s">
         <v>2388</v>
-      </c>
-      <c r="C848" s="3" t="s">
-        <v>2389</v>
       </c>
     </row>
     <row r="849" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A849" s="4" t="s">
+        <v>2390</v>
+      </c>
+      <c r="B849" s="5" t="s">
+        <v>2389</v>
+      </c>
+      <c r="C849" s="3" t="s">
         <v>2391</v>
-      </c>
-      <c r="B849" s="5" t="s">
-        <v>2390</v>
-      </c>
-      <c r="C849" s="3" t="s">
-        <v>2392</v>
       </c>
     </row>
     <row r="850" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A850" s="4" t="s">
+        <v>2392</v>
+      </c>
+      <c r="B850" s="5" t="s">
         <v>2393</v>
       </c>
-      <c r="B850" s="5" t="s">
+      <c r="C850" s="3" t="s">
         <v>2394</v>
-      </c>
-      <c r="C850" s="3" t="s">
-        <v>2395</v>
       </c>
     </row>
     <row r="851" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A851" s="4" t="s">
+        <v>2395</v>
+      </c>
+      <c r="B851" s="5" t="s">
         <v>2396</v>
       </c>
-      <c r="B851" s="5" t="s">
+      <c r="C851" s="3" t="s">
         <v>2397</v>
-      </c>
-      <c r="C851" s="3" t="s">
-        <v>2398</v>
       </c>
     </row>
     <row r="852" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A852" s="4" t="s">
-        <v>2401</v>
+        <v>2400</v>
       </c>
       <c r="B852" s="5" t="s">
-        <v>2440</v>
+        <v>2439</v>
       </c>
       <c r="C852" s="3" t="s">
         <v>1898</v>
@@ -31987,728 +31988,728 @@
     </row>
     <row r="853" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A853" s="4" t="s">
+        <v>2401</v>
+      </c>
+      <c r="B853" s="5" t="s">
+        <v>2440</v>
+      </c>
+      <c r="C853" s="3" t="s">
         <v>2402</v>
-      </c>
-      <c r="B853" s="5" t="s">
-        <v>2441</v>
-      </c>
-      <c r="C853" s="3" t="s">
-        <v>2403</v>
       </c>
     </row>
     <row r="854" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A854" s="4" t="s">
+        <v>2403</v>
+      </c>
+      <c r="B854" s="5" t="s">
+        <v>2441</v>
+      </c>
+      <c r="C854" s="3" t="s">
         <v>2404</v>
-      </c>
-      <c r="B854" s="5" t="s">
-        <v>2442</v>
-      </c>
-      <c r="C854" s="3" t="s">
-        <v>2405</v>
       </c>
     </row>
     <row r="855" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A855" s="4" t="s">
+        <v>2405</v>
+      </c>
+      <c r="B855" s="5" t="s">
+        <v>2442</v>
+      </c>
+      <c r="C855" s="3" t="s">
         <v>2406</v>
-      </c>
-      <c r="B855" s="5" t="s">
-        <v>2443</v>
-      </c>
-      <c r="C855" s="3" t="s">
-        <v>2407</v>
       </c>
     </row>
     <row r="856" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A856" s="4" t="s">
+        <v>2408</v>
+      </c>
+      <c r="B856" s="5" t="s">
+        <v>2443</v>
+      </c>
+      <c r="C856" s="3" t="s">
         <v>2409</v>
-      </c>
-      <c r="B856" s="5" t="s">
-        <v>2444</v>
-      </c>
-      <c r="C856" s="3" t="s">
-        <v>2410</v>
       </c>
     </row>
     <row r="857" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A857" s="4" t="s">
-        <v>2408</v>
+        <v>2407</v>
       </c>
       <c r="B857" s="5" t="s">
-        <v>2445</v>
+        <v>2444</v>
       </c>
       <c r="C857" s="3" t="s">
-        <v>2411</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="858" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A858" s="4" t="s">
+        <v>2411</v>
+      </c>
+      <c r="B858" s="5" t="s">
+        <v>2445</v>
+      </c>
+      <c r="C858" s="3" t="s">
         <v>2412</v>
-      </c>
-      <c r="B858" s="5" t="s">
-        <v>2446</v>
-      </c>
-      <c r="C858" s="3" t="s">
-        <v>2413</v>
       </c>
     </row>
     <row r="859" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A859" s="4" t="s">
+        <v>2413</v>
+      </c>
+      <c r="B859" s="5" t="s">
+        <v>2446</v>
+      </c>
+      <c r="C859" s="3" t="s">
         <v>2414</v>
-      </c>
-      <c r="B859" s="5" t="s">
-        <v>2447</v>
-      </c>
-      <c r="C859" s="3" t="s">
-        <v>2415</v>
       </c>
     </row>
     <row r="860" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A860" s="4" t="s">
+        <v>2415</v>
+      </c>
+      <c r="B860" s="5" t="s">
+        <v>2447</v>
+      </c>
+      <c r="C860" s="3" t="s">
         <v>2416</v>
-      </c>
-      <c r="B860" s="5" t="s">
-        <v>2448</v>
-      </c>
-      <c r="C860" s="3" t="s">
-        <v>2417</v>
       </c>
     </row>
     <row r="861" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A861" s="4" t="s">
-        <v>2399</v>
+        <v>2398</v>
       </c>
       <c r="B861" s="5" t="s">
-        <v>2449</v>
+        <v>2448</v>
       </c>
       <c r="C861" s="3" t="s">
-        <v>2418</v>
+        <v>2417</v>
       </c>
     </row>
     <row r="862" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A862" s="4" t="s">
-        <v>2400</v>
+        <v>2399</v>
       </c>
       <c r="B862" s="5" t="s">
-        <v>2450</v>
+        <v>2449</v>
       </c>
       <c r="C862" s="3" t="s">
-        <v>2424</v>
+        <v>2423</v>
       </c>
     </row>
     <row r="863" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A863" s="4" t="s">
-        <v>2425</v>
+        <v>2424</v>
       </c>
       <c r="B863" s="5" t="s">
-        <v>2451</v>
+        <v>2450</v>
       </c>
       <c r="C863" s="3" t="s">
-        <v>2419</v>
+        <v>2418</v>
       </c>
     </row>
     <row r="864" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A864" s="4" t="s">
-        <v>2426</v>
+        <v>2425</v>
       </c>
       <c r="B864" s="5" t="s">
-        <v>2452</v>
+        <v>2451</v>
       </c>
       <c r="C864" s="3" t="s">
-        <v>2420</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="865" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A865" s="4" t="s">
-        <v>2427</v>
+        <v>2426</v>
       </c>
       <c r="B865" s="5" t="s">
-        <v>2453</v>
+        <v>2452</v>
       </c>
       <c r="C865" s="3" t="s">
-        <v>2421</v>
+        <v>2420</v>
       </c>
     </row>
     <row r="866" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A866" s="4" t="s">
-        <v>2428</v>
+        <v>2427</v>
       </c>
       <c r="B866" s="5" t="s">
-        <v>2454</v>
+        <v>2453</v>
       </c>
       <c r="C866" s="3" t="s">
-        <v>2422</v>
+        <v>2421</v>
       </c>
     </row>
     <row r="867" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A867" s="4" t="s">
+        <v>2428</v>
+      </c>
+      <c r="B867" s="5" t="s">
+        <v>2454</v>
+      </c>
+      <c r="C867" s="3" t="s">
         <v>2429</v>
-      </c>
-      <c r="B867" s="5" t="s">
-        <v>2455</v>
-      </c>
-      <c r="C867" s="3" t="s">
-        <v>2430</v>
       </c>
     </row>
     <row r="868" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A868" s="4" t="s">
-        <v>2431</v>
+        <v>2430</v>
       </c>
       <c r="B868" s="5" t="s">
-        <v>2456</v>
+        <v>2455</v>
       </c>
       <c r="C868" s="3" t="s">
-        <v>2423</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="869" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A869" s="4" t="s">
+        <v>2431</v>
+      </c>
+      <c r="B869" s="5" t="s">
+        <v>2456</v>
+      </c>
+      <c r="C869" s="3" t="s">
         <v>2432</v>
-      </c>
-      <c r="B869" s="5" t="s">
-        <v>2457</v>
-      </c>
-      <c r="C869" s="3" t="s">
-        <v>2433</v>
       </c>
     </row>
     <row r="870" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A870" s="4" t="s">
+        <v>2433</v>
+      </c>
+      <c r="B870" s="5" t="s">
+        <v>2457</v>
+      </c>
+      <c r="C870" s="3" t="s">
         <v>2434</v>
-      </c>
-      <c r="B870" s="5" t="s">
-        <v>2458</v>
-      </c>
-      <c r="C870" s="3" t="s">
-        <v>2435</v>
       </c>
     </row>
     <row r="871" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A871" s="4" t="s">
+        <v>2435</v>
+      </c>
+      <c r="B871" s="5" t="s">
+        <v>2458</v>
+      </c>
+      <c r="C871" s="3" t="s">
         <v>2436</v>
-      </c>
-      <c r="B871" s="5" t="s">
-        <v>2459</v>
-      </c>
-      <c r="C871" s="3" t="s">
-        <v>2437</v>
       </c>
     </row>
     <row r="872" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A872" s="4" t="s">
+        <v>2437</v>
+      </c>
+      <c r="B872" s="5" t="s">
+        <v>2459</v>
+      </c>
+      <c r="C872" s="3" t="s">
         <v>2438</v>
-      </c>
-      <c r="B872" s="5" t="s">
-        <v>2460</v>
-      </c>
-      <c r="C872" s="3" t="s">
-        <v>2439</v>
       </c>
     </row>
     <row r="873" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A873" s="4" t="s">
+        <v>2460</v>
+      </c>
+      <c r="B873" s="5" t="s">
+        <v>2462</v>
+      </c>
+      <c r="C873" s="3" t="s">
         <v>2461</v>
-      </c>
-      <c r="B873" s="5" t="s">
-        <v>2463</v>
-      </c>
-      <c r="C873" s="3" t="s">
-        <v>2462</v>
       </c>
     </row>
     <row r="874" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A874" s="4" t="s">
+        <v>2463</v>
+      </c>
+      <c r="B874" s="5" t="s">
         <v>2464</v>
       </c>
-      <c r="B874" s="5" t="s">
+      <c r="C874" s="3" t="s">
         <v>2465</v>
-      </c>
-      <c r="C874" s="3" t="s">
-        <v>2466</v>
       </c>
     </row>
     <row r="875" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A875" s="4" t="s">
-        <v>2467</v>
+        <v>2466</v>
       </c>
       <c r="B875" s="5" t="s">
-        <v>2487</v>
+        <v>2486</v>
       </c>
       <c r="C875" s="3" t="s">
-        <v>2507</v>
+        <v>2506</v>
       </c>
     </row>
     <row r="876" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A876" s="4" t="s">
-        <v>2468</v>
+        <v>2467</v>
       </c>
       <c r="B876" s="5" t="s">
-        <v>2488</v>
+        <v>2487</v>
       </c>
       <c r="C876" s="3" t="s">
-        <v>2508</v>
+        <v>2507</v>
       </c>
     </row>
     <row r="877" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A877" s="4" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="B877" s="5" t="s">
-        <v>2489</v>
+        <v>2488</v>
       </c>
       <c r="C877" s="3" t="s">
-        <v>2509</v>
+        <v>2508</v>
       </c>
     </row>
     <row r="878" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A878" s="4" t="s">
-        <v>2470</v>
+        <v>2469</v>
       </c>
       <c r="B878" s="5" t="s">
-        <v>2490</v>
+        <v>2489</v>
       </c>
       <c r="C878" s="3" t="s">
-        <v>2510</v>
+        <v>2509</v>
       </c>
     </row>
     <row r="879" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A879" s="4" t="s">
-        <v>2471</v>
+        <v>2470</v>
       </c>
       <c r="B879" s="5" t="s">
-        <v>2491</v>
+        <v>2490</v>
       </c>
       <c r="C879" s="3" t="s">
-        <v>2511</v>
+        <v>2510</v>
       </c>
     </row>
     <row r="880" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A880" s="4" t="s">
-        <v>2472</v>
+        <v>2471</v>
       </c>
       <c r="B880" s="5" t="s">
-        <v>2492</v>
+        <v>2491</v>
       </c>
       <c r="C880" s="3" t="s">
-        <v>2512</v>
+        <v>2511</v>
       </c>
     </row>
     <row r="881" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A881" s="4" t="s">
-        <v>2473</v>
+        <v>2472</v>
       </c>
       <c r="B881" s="5" t="s">
-        <v>2493</v>
+        <v>2492</v>
       </c>
       <c r="C881" s="3" t="s">
-        <v>2513</v>
+        <v>2512</v>
       </c>
     </row>
     <row r="882" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A882" s="4" t="s">
-        <v>2474</v>
+        <v>2473</v>
       </c>
       <c r="B882" s="5" t="s">
-        <v>2494</v>
+        <v>2493</v>
       </c>
       <c r="C882" s="3" t="s">
-        <v>2514</v>
+        <v>2513</v>
       </c>
     </row>
     <row r="883" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A883" s="4" t="s">
-        <v>2475</v>
+        <v>2474</v>
       </c>
       <c r="B883" s="5" t="s">
-        <v>2495</v>
+        <v>2494</v>
       </c>
       <c r="C883" s="3" t="s">
-        <v>2515</v>
+        <v>2514</v>
       </c>
     </row>
     <row r="884" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A884" s="4" t="s">
-        <v>2476</v>
+        <v>2475</v>
       </c>
       <c r="B884" s="5" t="s">
-        <v>2496</v>
+        <v>2495</v>
       </c>
       <c r="C884" s="3" t="s">
-        <v>2516</v>
+        <v>2515</v>
       </c>
     </row>
     <row r="885" spans="1:3" ht="285" x14ac:dyDescent="0.4">
       <c r="A885" s="4" t="s">
+        <v>2537</v>
+      </c>
+      <c r="B885" s="5" t="s">
         <v>2538</v>
       </c>
-      <c r="B885" s="5" t="s">
+      <c r="C885" s="3" t="s">
         <v>2539</v>
-      </c>
-      <c r="C885" s="3" t="s">
-        <v>2540</v>
       </c>
     </row>
     <row r="886" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A886" s="4" t="s">
-        <v>2477</v>
+        <v>2476</v>
       </c>
       <c r="B886" s="5" t="s">
-        <v>2497</v>
+        <v>2496</v>
       </c>
       <c r="C886" s="3" t="s">
-        <v>2497</v>
+        <v>2496</v>
       </c>
     </row>
     <row r="887" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A887" s="4" t="s">
-        <v>2478</v>
+        <v>2477</v>
       </c>
       <c r="B887" s="5" t="s">
-        <v>2498</v>
+        <v>2497</v>
       </c>
       <c r="C887" s="3" t="s">
-        <v>2517</v>
+        <v>2516</v>
       </c>
     </row>
     <row r="888" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A888" s="4" t="s">
-        <v>2479</v>
+        <v>2478</v>
       </c>
       <c r="B888" s="5" t="s">
-        <v>2499</v>
+        <v>2498</v>
       </c>
       <c r="C888" s="3" t="s">
-        <v>2518</v>
+        <v>2517</v>
       </c>
     </row>
     <row r="889" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A889" s="4" t="s">
-        <v>2480</v>
+        <v>2479</v>
       </c>
       <c r="B889" s="5" t="s">
-        <v>2500</v>
+        <v>2499</v>
       </c>
       <c r="C889" s="3" t="s">
-        <v>2519</v>
+        <v>2518</v>
       </c>
     </row>
     <row r="890" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A890" s="4" t="s">
-        <v>2481</v>
+        <v>2480</v>
       </c>
       <c r="B890" s="5" t="s">
-        <v>2501</v>
+        <v>2500</v>
       </c>
       <c r="C890" s="3" t="s">
-        <v>2501</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="891" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A891" s="4" t="s">
-        <v>2482</v>
+        <v>2481</v>
       </c>
       <c r="B891" s="5" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="C891" s="3" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
     </row>
     <row r="892" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A892" s="4" t="s">
-        <v>2483</v>
+        <v>2482</v>
       </c>
       <c r="B892" s="5" t="s">
-        <v>2503</v>
+        <v>2502</v>
       </c>
       <c r="C892" s="3" t="s">
-        <v>2503</v>
+        <v>2502</v>
       </c>
     </row>
     <row r="893" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A893" s="4" t="s">
-        <v>2484</v>
+        <v>2483</v>
       </c>
       <c r="B893" s="5" t="s">
-        <v>2504</v>
+        <v>2503</v>
       </c>
       <c r="C893" s="3" t="s">
-        <v>2504</v>
+        <v>2503</v>
       </c>
     </row>
     <row r="894" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A894" s="4" t="s">
-        <v>2485</v>
+        <v>2484</v>
       </c>
       <c r="B894" s="5" t="s">
-        <v>2505</v>
+        <v>2504</v>
       </c>
       <c r="C894" s="3" t="s">
-        <v>2505</v>
+        <v>2504</v>
       </c>
     </row>
     <row r="895" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A895" s="4" t="s">
-        <v>2486</v>
+        <v>2485</v>
       </c>
       <c r="B895" s="5" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="C895" s="3" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
     </row>
     <row r="896" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A896" s="4" t="s">
-        <v>2520</v>
+        <v>2519</v>
       </c>
       <c r="B896" s="5" t="s">
-        <v>2522</v>
+        <v>2521</v>
       </c>
       <c r="C896" s="3" t="s">
-        <v>2524</v>
+        <v>2523</v>
       </c>
     </row>
     <row r="897" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A897" s="4" t="s">
-        <v>2521</v>
+        <v>2520</v>
       </c>
       <c r="B897" s="5" t="s">
-        <v>2523</v>
+        <v>2522</v>
       </c>
       <c r="C897" s="3" t="s">
-        <v>2525</v>
+        <v>2524</v>
       </c>
     </row>
     <row r="898" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A898" s="4" t="s">
+        <v>2525</v>
+      </c>
+      <c r="B898" s="5" t="s">
+        <v>2527</v>
+      </c>
+      <c r="C898" s="3" t="s">
         <v>2526</v>
-      </c>
-      <c r="B898" s="5" t="s">
-        <v>2528</v>
-      </c>
-      <c r="C898" s="3" t="s">
-        <v>2527</v>
       </c>
     </row>
     <row r="899" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A899" s="4" t="s">
+        <v>2528</v>
+      </c>
+      <c r="B899" s="5" t="s">
         <v>2529</v>
       </c>
-      <c r="B899" s="5" t="s">
+      <c r="C899" s="3" t="s">
         <v>2530</v>
-      </c>
-      <c r="C899" s="3" t="s">
-        <v>2531</v>
       </c>
     </row>
     <row r="900" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A900" s="4" t="s">
+        <v>2531</v>
+      </c>
+      <c r="B900" s="5" t="s">
         <v>2532</v>
       </c>
-      <c r="B900" s="5" t="s">
+      <c r="C900" s="3" t="s">
         <v>2533</v>
-      </c>
-      <c r="C900" s="3" t="s">
-        <v>2534</v>
       </c>
     </row>
     <row r="901" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A901" s="4" t="s">
+        <v>2535</v>
+      </c>
+      <c r="B901" s="5" t="s">
+        <v>2534</v>
+      </c>
+      <c r="C901" s="3" t="s">
         <v>2536</v>
-      </c>
-      <c r="B901" s="5" t="s">
-        <v>2535</v>
-      </c>
-      <c r="C901" s="3" t="s">
-        <v>2537</v>
       </c>
     </row>
     <row r="902" spans="1:3" ht="38" x14ac:dyDescent="0.4">
       <c r="A902" s="4" t="s">
+        <v>2540</v>
+      </c>
+      <c r="B902" s="5" t="s">
+        <v>2542</v>
+      </c>
+      <c r="C902" s="3" t="s">
         <v>2541</v>
-      </c>
-      <c r="B902" s="5" t="s">
-        <v>2543</v>
-      </c>
-      <c r="C902" s="3" t="s">
-        <v>2542</v>
       </c>
     </row>
     <row r="903" spans="1:3" ht="38" x14ac:dyDescent="0.4">
       <c r="A903" s="4" t="s">
+        <v>2543</v>
+      </c>
+      <c r="B903" s="5" t="s">
+        <v>2545</v>
+      </c>
+      <c r="C903" s="3" t="s">
         <v>2544</v>
-      </c>
-      <c r="B903" s="5" t="s">
-        <v>2546</v>
-      </c>
-      <c r="C903" s="3" t="s">
-        <v>2545</v>
       </c>
     </row>
     <row r="904" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A904" s="4" t="s">
+        <v>2547</v>
+      </c>
+      <c r="B904" s="5" t="s">
+        <v>2546</v>
+      </c>
+      <c r="C904" s="3" t="s">
         <v>2548</v>
-      </c>
-      <c r="B904" s="5" t="s">
-        <v>2547</v>
-      </c>
-      <c r="C904" s="3" t="s">
-        <v>2549</v>
       </c>
     </row>
     <row r="905" spans="1:3" ht="38" x14ac:dyDescent="0.4">
       <c r="A905" s="4" t="s">
+        <v>2550</v>
+      </c>
+      <c r="B905" s="5" t="s">
         <v>2551</v>
       </c>
-      <c r="B905" s="5" t="s">
+      <c r="C905" s="3" t="s">
         <v>2552</v>
-      </c>
-      <c r="C905" s="3" t="s">
-        <v>2553</v>
       </c>
     </row>
     <row r="906" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A906" s="4" t="s">
+        <v>2553</v>
+      </c>
+      <c r="B906" s="5" t="s">
+        <v>2555</v>
+      </c>
+      <c r="C906" s="3" t="s">
         <v>2554</v>
-      </c>
-      <c r="B906" s="5" t="s">
-        <v>2556</v>
-      </c>
-      <c r="C906" s="3" t="s">
-        <v>2555</v>
       </c>
     </row>
     <row r="907" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A907" s="4" t="s">
-        <v>2560</v>
+        <v>2559</v>
       </c>
       <c r="B907" s="5" t="s">
-        <v>2563</v>
+        <v>2562</v>
       </c>
       <c r="C907" s="3" t="s">
-        <v>2557</v>
+        <v>2556</v>
       </c>
     </row>
     <row r="908" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A908" s="4" t="s">
-        <v>2561</v>
+        <v>2560</v>
       </c>
       <c r="B908" s="5" t="s">
-        <v>2564</v>
+        <v>2563</v>
       </c>
       <c r="C908" s="3" t="s">
-        <v>2558</v>
+        <v>2557</v>
       </c>
     </row>
     <row r="909" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A909" s="4" t="s">
-        <v>2562</v>
+        <v>2561</v>
       </c>
       <c r="B909" s="5" t="s">
-        <v>2565</v>
+        <v>2564</v>
       </c>
       <c r="C909" s="3" t="s">
-        <v>2559</v>
+        <v>2558</v>
       </c>
     </row>
     <row r="910" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A910" s="4" t="s">
-        <v>2569</v>
+        <v>2568</v>
       </c>
       <c r="B910" s="5" t="s">
-        <v>2572</v>
+        <v>2571</v>
       </c>
       <c r="C910" s="3" t="s">
-        <v>2566</v>
+        <v>2565</v>
       </c>
     </row>
     <row r="911" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A911" s="4" t="s">
-        <v>2570</v>
+        <v>2569</v>
       </c>
       <c r="B911" s="5" t="s">
-        <v>2573</v>
+        <v>2572</v>
       </c>
       <c r="C911" s="3" t="s">
-        <v>2567</v>
+        <v>2566</v>
       </c>
     </row>
     <row r="912" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A912" s="4" t="s">
-        <v>2571</v>
+        <v>2570</v>
       </c>
       <c r="B912" s="5" t="s">
-        <v>2574</v>
+        <v>2573</v>
       </c>
       <c r="C912" s="3" t="s">
-        <v>2568</v>
+        <v>2567</v>
       </c>
     </row>
     <row r="913" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A913" s="4" t="s">
+        <v>2574</v>
+      </c>
+      <c r="B913" s="5" t="s">
         <v>2575</v>
       </c>
-      <c r="B913" s="5" t="s">
+      <c r="C913" s="3" t="s">
         <v>2576</v>
-      </c>
-      <c r="C913" s="3" t="s">
-        <v>2577</v>
       </c>
     </row>
     <row r="914" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A914" s="4" t="s">
-        <v>2578</v>
+        <v>2577</v>
       </c>
       <c r="B914" s="5" t="s">
+        <v>2575</v>
+      </c>
+      <c r="C914" s="3" t="s">
         <v>2576</v>
-      </c>
-      <c r="C914" s="3" t="s">
-        <v>2577</v>
       </c>
     </row>
     <row r="915" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A915" s="4" t="s">
+        <v>2578</v>
+      </c>
+      <c r="B915" s="5" t="s">
+        <v>2580</v>
+      </c>
+      <c r="C915" s="3" t="s">
         <v>2579</v>
-      </c>
-      <c r="B915" s="5" t="s">
-        <v>2581</v>
-      </c>
-      <c r="C915" s="3" t="s">
-        <v>2580</v>
       </c>
     </row>
     <row r="916" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A916" s="4" t="s">
+        <v>2582</v>
+      </c>
+      <c r="B916" s="5" t="s">
         <v>2583</v>
       </c>
-      <c r="B916" s="5" t="s">
-        <v>2584</v>
-      </c>
       <c r="C916" s="3" t="s">
-        <v>2582</v>
+        <v>2581</v>
       </c>
     </row>
     <row r="917" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A917" s="4" t="s">
+        <v>2584</v>
+      </c>
+      <c r="B917" s="5" t="s">
+        <v>2586</v>
+      </c>
+      <c r="C917" s="3" t="s">
         <v>2585</v>
-      </c>
-      <c r="B917" s="5" t="s">
-        <v>2587</v>
-      </c>
-      <c r="C917" s="3" t="s">
-        <v>2586</v>
       </c>
     </row>
     <row r="918" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A918" s="4" t="s">
+        <v>2588</v>
+      </c>
+      <c r="B918" s="5" t="s">
         <v>2589</v>
       </c>
-      <c r="B918" s="5" t="s">
-        <v>2590</v>
-      </c>
       <c r="C918" s="3" t="s">
-        <v>2588</v>
+        <v>2587</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add group and search function
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80AA0536-FF3B-4C9E-88B6-8E7DE506D008}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2F58980-1419-450D-B0B1-908E24B00EC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2240" yWindow="2240" windowWidth="31590" windowHeight="15280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2748" uniqueCount="2591">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2787" uniqueCount="2630">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -22206,17 +22206,208 @@
     <t>双击打开地图文件时，从地图目录加载资源文件</t>
   </si>
   <si>
+    <t>Options.EnableVeinholeLogic</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Display remapable colors of overlays</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>启用泰伯利亚藤蔓（蔓孔）逻辑</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>Enable veinhole logic</t>
-  </si>
-  <si>
-    <t>Options.EnableVeinholeLogic</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>启用泰伯利亚藤蔓（蔓孔）逻辑</t>
-  </si>
-  <si>
-    <t>Display remapable colors of overlays</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>GridObjectViewer.Group</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Group:</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>GridObjectViewer.Search</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Search:</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>GridObjectViewer.AllInfantry</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>All infantries</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>GridObjectViewer.AllVehicle</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>All vehicles</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>GridObjectViewer.AllAircraft</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>All aircrafts</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>GridObjectViewer.AllBuilding</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>All buildings</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>GridObjectViewer.AllTerrain</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>All terrain types</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>GridObjectViewer.AllSmudge</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>All smudges</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>GridObjectViewer.All</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>All objects</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>对象分组:</t>
+  </si>
+  <si>
+    <t>搜索:</t>
+  </si>
+  <si>
+    <t>所有步兵</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>所有车辆</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>所有飞行器</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>所有建筑</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>所有地形对象</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>所有污染</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>所有对象</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>TabPages.GridObjectViewer</t>
+  </si>
+  <si>
+    <t>Object Viewer</t>
+  </si>
+  <si>
+    <t>对象查看器</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Options.GridObjectViewer.LoadEditorCategory</t>
+  </si>
+  <si>
+    <t>Options.GridObjectViewer.LoadForceSides</t>
+  </si>
+  <si>
+    <r>
+      <t>根据对象的</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="15"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>EditorCategory</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="15"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>在对象查看器中分类</t>
+    </r>
+  </si>
+  <si>
+    <t>Classify objects in the object viewer based on their EditCategory</t>
+  </si>
+  <si>
+    <r>
+      <t>根据对象的</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="15"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>ForceSides</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="15"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>在对象查看器中分类</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Classify objects in the object viewer based on their ForceSides</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>GridObjectViewer.CurrentSelect</t>
+  </si>
+  <si>
+    <t>当前选择:</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Current:</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -22623,7 +22814,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C918"/>
+  <dimension ref="A1:C942"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="4" customWidth="1"/>
@@ -31807,7 +31998,7 @@
         <v>2356</v>
       </c>
       <c r="C836" s="3" t="s">
-        <v>2590</v>
+        <v>2588</v>
       </c>
     </row>
     <row r="837" spans="1:3" x14ac:dyDescent="0.4">
@@ -32701,16 +32892,203 @@
         <v>2585</v>
       </c>
     </row>
-    <row r="918" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="918" spans="1:3" ht="19" x14ac:dyDescent="0.4">
       <c r="A918" s="4" t="s">
-        <v>2588</v>
-      </c>
-      <c r="B918" s="5" t="s">
+        <v>2587</v>
+      </c>
+      <c r="B918" s="4" t="s">
         <v>2589</v>
       </c>
-      <c r="C918" s="3" t="s">
-        <v>2587</v>
-      </c>
+      <c r="C918" s="4" t="s">
+        <v>2590</v>
+      </c>
+    </row>
+    <row r="919" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A919" s="4" t="s">
+        <v>2591</v>
+      </c>
+      <c r="B919" s="5" t="s">
+        <v>2609</v>
+      </c>
+      <c r="C919" s="4" t="s">
+        <v>2592</v>
+      </c>
+    </row>
+    <row r="920" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A920" s="4" t="s">
+        <v>2593</v>
+      </c>
+      <c r="B920" s="5" t="s">
+        <v>2610</v>
+      </c>
+      <c r="C920" s="4" t="s">
+        <v>2594</v>
+      </c>
+    </row>
+    <row r="921" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A921" s="4" t="s">
+        <v>2627</v>
+      </c>
+      <c r="B921" s="5" t="s">
+        <v>2628</v>
+      </c>
+      <c r="C921" s="4" t="s">
+        <v>2629</v>
+      </c>
+    </row>
+    <row r="922" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A922" s="4" t="s">
+        <v>2595</v>
+      </c>
+      <c r="B922" s="5" t="s">
+        <v>2611</v>
+      </c>
+      <c r="C922" s="4" t="s">
+        <v>2596</v>
+      </c>
+    </row>
+    <row r="923" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A923" s="4" t="s">
+        <v>2597</v>
+      </c>
+      <c r="B923" s="5" t="s">
+        <v>2612</v>
+      </c>
+      <c r="C923" s="4" t="s">
+        <v>2598</v>
+      </c>
+    </row>
+    <row r="924" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A924" s="4" t="s">
+        <v>2599</v>
+      </c>
+      <c r="B924" s="5" t="s">
+        <v>2613</v>
+      </c>
+      <c r="C924" s="4" t="s">
+        <v>2600</v>
+      </c>
+    </row>
+    <row r="925" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A925" s="4" t="s">
+        <v>2601</v>
+      </c>
+      <c r="B925" s="5" t="s">
+        <v>2614</v>
+      </c>
+      <c r="C925" s="4" t="s">
+        <v>2602</v>
+      </c>
+    </row>
+    <row r="926" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A926" s="4" t="s">
+        <v>2603</v>
+      </c>
+      <c r="B926" s="5" t="s">
+        <v>2615</v>
+      </c>
+      <c r="C926" s="4" t="s">
+        <v>2604</v>
+      </c>
+    </row>
+    <row r="927" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A927" s="4" t="s">
+        <v>2605</v>
+      </c>
+      <c r="B927" s="5" t="s">
+        <v>2616</v>
+      </c>
+      <c r="C927" s="4" t="s">
+        <v>2606</v>
+      </c>
+    </row>
+    <row r="928" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A928" s="4" t="s">
+        <v>2607</v>
+      </c>
+      <c r="B928" s="5" t="s">
+        <v>2617</v>
+      </c>
+      <c r="C928" s="4" t="s">
+        <v>2608</v>
+      </c>
+    </row>
+    <row r="929" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A929" s="4" t="s">
+        <v>2618</v>
+      </c>
+      <c r="B929" s="5" t="s">
+        <v>2620</v>
+      </c>
+      <c r="C929" s="4" t="s">
+        <v>2619</v>
+      </c>
+    </row>
+    <row r="930" spans="1:3" ht="38" x14ac:dyDescent="0.4">
+      <c r="A930" s="4" t="s">
+        <v>2621</v>
+      </c>
+      <c r="B930" s="5" t="s">
+        <v>2623</v>
+      </c>
+      <c r="C930" s="4" t="s">
+        <v>2624</v>
+      </c>
+    </row>
+    <row r="931" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A931" s="4" t="s">
+        <v>2622</v>
+      </c>
+      <c r="B931" s="5" t="s">
+        <v>2625</v>
+      </c>
+      <c r="C931" s="4" t="s">
+        <v>2626</v>
+      </c>
+    </row>
+    <row r="932" spans="1:3" ht="19" x14ac:dyDescent="0.4">
+      <c r="B932" s="4"/>
+      <c r="C932" s="4"/>
+    </row>
+    <row r="933" spans="1:3" ht="19" x14ac:dyDescent="0.4">
+      <c r="B933" s="4"/>
+      <c r="C933" s="4"/>
+    </row>
+    <row r="934" spans="1:3" ht="19" x14ac:dyDescent="0.4">
+      <c r="B934" s="4"/>
+      <c r="C934" s="4"/>
+    </row>
+    <row r="935" spans="1:3" ht="19" x14ac:dyDescent="0.4">
+      <c r="B935" s="4"/>
+      <c r="C935" s="4"/>
+    </row>
+    <row r="936" spans="1:3" ht="19" x14ac:dyDescent="0.4">
+      <c r="B936" s="4"/>
+      <c r="C936" s="4"/>
+    </row>
+    <row r="937" spans="1:3" ht="19" x14ac:dyDescent="0.4">
+      <c r="B937" s="4"/>
+      <c r="C937" s="4"/>
+    </row>
+    <row r="938" spans="1:3" ht="19" x14ac:dyDescent="0.4">
+      <c r="B938" s="4"/>
+      <c r="C938" s="4"/>
+    </row>
+    <row r="939" spans="1:3" ht="19" x14ac:dyDescent="0.4">
+      <c r="B939" s="4"/>
+      <c r="C939" s="4"/>
+    </row>
+    <row r="940" spans="1:3" ht="19" x14ac:dyDescent="0.4">
+      <c r="B940" s="4"/>
+      <c r="C940" s="4"/>
+    </row>
+    <row r="941" spans="1:3" ht="19" x14ac:dyDescent="0.4">
+      <c r="B941" s="4"/>
+      <c r="C941" s="4"/>
+    </row>
+    <row r="942" spans="1:3" ht="19" x14ac:dyDescent="0.4">
+      <c r="B942" s="4"/>
+      <c r="C942" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
object viewer supports overlays
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95510E20-EB25-426A-98A9-E1F8BF07D2DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B96FDB7-868A-40F5-8C4F-22AE83C530B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2240" yWindow="2240" windowWidth="31590" windowHeight="15280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2829" uniqueCount="2683">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2853" uniqueCount="2707">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -23289,6 +23289,86 @@
   </si>
   <si>
     <t>Center</t>
+  </si>
+  <si>
+    <t>地表类型: %#x, 高度 %d /</t>
+  </si>
+  <si>
+    <t>覆盖物: %#x, 覆盖物数据: %#x /</t>
+  </si>
+  <si>
+    <t>建筑: ID %d, %s (%s, %s) /</t>
+  </si>
+  <si>
+    <t>车辆: ID %d, %s (%s, %s) /</t>
+  </si>
+  <si>
+    <t>飞行器: ID %d, %s (%s, %s) /</t>
+  </si>
+  <si>
+    <t>步兵: ID %d, %s (%s, %s) /</t>
+  </si>
+  <si>
+    <t>单元标记: %s (%s) /</t>
+  </si>
+  <si>
+    <t>StatusBarText7</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>StatusBarText6</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>StatusBarText5</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>StatusBarText4</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>StatusBarText3</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>StatusBarText2</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>StatusBarText1</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Terrain type: %#x, height %d /</t>
+  </si>
+  <si>
+    <t>Overlay: %#x, OverlayData %#x /</t>
+  </si>
+  <si>
+    <t>Structure: ID %d, %s (%s, %s) /</t>
+  </si>
+  <si>
+    <t>Vehicle: ID %d, %s (%s, %s) /</t>
+  </si>
+  <si>
+    <t>Aircraft: ID %d, %s (%s, %s) /</t>
+  </si>
+  <si>
+    <t>Infantry: ID %d, %s (%s, %s) /</t>
+  </si>
+  <si>
+    <t>CellTag: %s (%s) /</t>
+  </si>
+  <si>
+    <t>GridObjectViewer.OverlayText</t>
+  </si>
+  <si>
+    <t>索引: %d, 覆盖物数据: %d</t>
+  </si>
+  <si>
+    <t>Index: %d, OverlayData: %d</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -23682,7 +23762,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C945"/>
+  <dimension ref="A1:C953"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -34068,8 +34148,97 @@
         <v>2682</v>
       </c>
     </row>
+    <row r="946" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A946" s="3" t="s">
+        <v>2696</v>
+      </c>
+      <c r="B946" s="4" t="s">
+        <v>2683</v>
+      </c>
+      <c r="C946" s="3" t="s">
+        <v>2697</v>
+      </c>
+    </row>
+    <row r="947" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A947" s="3" t="s">
+        <v>2695</v>
+      </c>
+      <c r="B947" s="4" t="s">
+        <v>2684</v>
+      </c>
+      <c r="C947" s="3" t="s">
+        <v>2698</v>
+      </c>
+    </row>
+    <row r="948" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A948" s="3" t="s">
+        <v>2694</v>
+      </c>
+      <c r="B948" s="4" t="s">
+        <v>2685</v>
+      </c>
+      <c r="C948" s="3" t="s">
+        <v>2699</v>
+      </c>
+    </row>
+    <row r="949" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A949" s="3" t="s">
+        <v>2693</v>
+      </c>
+      <c r="B949" s="4" t="s">
+        <v>2686</v>
+      </c>
+      <c r="C949" s="3" t="s">
+        <v>2700</v>
+      </c>
+    </row>
+    <row r="950" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A950" s="3" t="s">
+        <v>2692</v>
+      </c>
+      <c r="B950" s="4" t="s">
+        <v>2687</v>
+      </c>
+      <c r="C950" s="3" t="s">
+        <v>2701</v>
+      </c>
+    </row>
+    <row r="951" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A951" s="3" t="s">
+        <v>2691</v>
+      </c>
+      <c r="B951" s="4" t="s">
+        <v>2688</v>
+      </c>
+      <c r="C951" s="3" t="s">
+        <v>2702</v>
+      </c>
+    </row>
+    <row r="952" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A952" s="3" t="s">
+        <v>2690</v>
+      </c>
+      <c r="B952" s="4" t="s">
+        <v>2689</v>
+      </c>
+      <c r="C952" s="3" t="s">
+        <v>2703</v>
+      </c>
+    </row>
+    <row r="953" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A953" s="3" t="s">
+        <v>2704</v>
+      </c>
+      <c r="B953" s="4" t="s">
+        <v>2705</v>
+      </c>
+      <c r="C953" s="3" t="s">
+        <v>2706</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add check for update function
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B96FDB7-868A-40F5-8C4F-22AE83C530B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EEC952D-FC7C-4416-9BDF-1DC55DBAAB11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2853" uniqueCount="2707">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2856" uniqueCount="2710">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -23369,6 +23369,16 @@
   <si>
     <t>Index: %d, OverlayData: %d</t>
     <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>NewVersionAvailable</t>
+  </si>
+  <si>
+    <t>发现新版本:</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>New version available:</t>
   </si>
 </sst>
 </file>
@@ -23762,7 +23772,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C953"/>
+  <dimension ref="A1:C954"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -34236,6 +34246,17 @@
         <v>2706</v>
       </c>
     </row>
+    <row r="954" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A954" s="3" t="s">
+        <v>2707</v>
+      </c>
+      <c r="B954" s="4" t="s">
+        <v>2708</v>
+      </c>
+      <c r="C954" s="3" t="s">
+        <v>2709</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
support display on second screen
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81FA97EA-A56C-4AC2-B5F4-D9CF7CEC6493}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AB06740-AF92-4831-B1CF-DF650C2FC295}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2859" uniqueCount="2713">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2862" uniqueCount="2716">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -23388,6 +23388,16 @@
   </si>
   <si>
     <t>Always assign the next incremental index when creating triggers and teams</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Options.SecondScreenSupport</t>
+  </si>
+  <si>
+    <t>Support displaying IsoView on non-primary screens (slower)</t>
+  </si>
+  <si>
+    <t>支持副屏显示绘图界面（轻微影响性能）</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -23782,7 +23792,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C955"/>
+  <dimension ref="A1:C956"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -34278,6 +34288,17 @@
         <v>2708</v>
       </c>
     </row>
+    <row r="956" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A956" s="3" t="s">
+        <v>2713</v>
+      </c>
+      <c r="B956" s="4" t="s">
+        <v>2715</v>
+      </c>
+      <c r="C956" s="3" t="s">
+        <v>2714</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add phobos script action 14004
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F193F983-4F94-44FC-B6BB-8CB645883D77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66B20F63-9F70-41A7-A477-333899E291FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2874" uniqueCount="2728">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2877" uniqueCount="2731">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -23439,6 +23439,16 @@
   </si>
   <si>
     <t>Circle Tool</t>
+  </si>
+  <si>
+    <t>MeasurementToolbox.LineSegment</t>
+  </si>
+  <si>
+    <t>线段(无文本)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Line Segment (no text)</t>
   </si>
 </sst>
 </file>
@@ -23832,7 +23842,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C960"/>
+  <dimension ref="A1:C961"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -34383,6 +34393,17 @@
         <v>2724</v>
       </c>
     </row>
+    <row r="961" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A961" s="3" t="s">
+        <v>2728</v>
+      </c>
+      <c r="B961" s="4" t="s">
+        <v>2729</v>
+      </c>
+      <c r="C961" s="3" t="s">
+        <v>2730</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
measurement toolbox support undo redo
display script path
fix object search bugs
display <player @ X> at bottom in trigger editor
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41765373-225A-464A-A5FF-9C8574C16A9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D6CDC4E-866B-4070-9390-002121C0E425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2660" yWindow="2660" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2880" uniqueCount="2734">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2883" uniqueCount="2737">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -23460,6 +23460,17 @@
   </si>
   <si>
     <t>根据污染/地形对象/覆盖物在物品浏览器中的分组在对象查看器中分类</t>
+  </si>
+  <si>
+    <t>ScriptTypesRenderPath</t>
+  </si>
+  <si>
+    <t>渲染路径</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Render path</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -23853,7 +23864,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C962"/>
+  <dimension ref="A1:C963"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -34426,6 +34437,17 @@
         <v>2731</v>
       </c>
     </row>
+    <row r="963" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A963" s="3" t="s">
+        <v>2734</v>
+      </c>
+      <c r="B963" s="4" t="s">
+        <v>2735</v>
+      </c>
+      <c r="C963" s="3" t="s">
+        <v>2736</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add ignore landtype button in terrain generator
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D6CDC4E-866B-4070-9390-002121C0E425}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12D141E8-64BD-4988-A75E-0DF043002BE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2660" yWindow="2660" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5940" yWindow="2730" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2883" uniqueCount="2737">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2886" uniqueCount="2740">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -23471,6 +23471,16 @@
   <si>
     <t>Render path</t>
     <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>忽视地表类型</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ignore Landtypes</t>
+  </si>
+  <si>
+    <t>CTerrainGenerator.IgnoreLandtypes</t>
   </si>
 </sst>
 </file>
@@ -23864,7 +23874,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C963"/>
+  <dimension ref="A1:C964"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -34448,6 +34458,17 @@
         <v>2736</v>
       </c>
     </row>
+    <row r="964" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A964" s="3" t="s">
+        <v>2739</v>
+      </c>
+      <c r="B964" s="4" t="s">
+        <v>2737</v>
+      </c>
+      <c r="C964" s="3" t="s">
+        <v>2738</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add missing translation in house dialog, fix random placement icon
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12D141E8-64BD-4988-A75E-0DF043002BE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{460C50B5-8CFB-4057-BA05-AF7DA47A98E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5940" yWindow="2730" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2886" uniqueCount="2740">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2895" uniqueCount="2749">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -23481,6 +23481,42 @@
   </si>
   <si>
     <t>CTerrainGenerator.IgnoreLandtypes</t>
+  </si>
+  <si>
+    <t>There are already houses in your map. You need to delete these first</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>No houses do exist, if you want to use houses, you should use Prepare houses before doing anything else.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Sorry this name is not available. %s is already used in the map file. You need to use another name.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>HouseDialog.NoHousesExist</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>HouseDialog.AlreadyHouses</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>HouseDialog.NotAvailable</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>地图还没有任何所属方。你需要使用标准所属方，或新建所属方。</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>地图已经存在所属方，要使用此功能，需要先删除它们。</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>所属方名称 %s 已经被使用，你需要换一个名字。</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -23874,7 +23910,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C964"/>
+  <dimension ref="A1:C967"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -34469,6 +34505,39 @@
         <v>2738</v>
       </c>
     </row>
+    <row r="965" spans="1:3" ht="38" x14ac:dyDescent="0.4">
+      <c r="A965" s="3" t="s">
+        <v>2743</v>
+      </c>
+      <c r="B965" s="4" t="s">
+        <v>2746</v>
+      </c>
+      <c r="C965" s="3" t="s">
+        <v>2741</v>
+      </c>
+    </row>
+    <row r="966" spans="1:3" ht="38" x14ac:dyDescent="0.4">
+      <c r="A966" s="3" t="s">
+        <v>2744</v>
+      </c>
+      <c r="B966" s="4" t="s">
+        <v>2747</v>
+      </c>
+      <c r="C966" s="3" t="s">
+        <v>2740</v>
+      </c>
+    </row>
+    <row r="967" spans="1:3" ht="38" x14ac:dyDescent="0.4">
+      <c r="A967" s="3" t="s">
+        <v>2745</v>
+      </c>
+      <c r="B967" s="4" t="s">
+        <v>2748</v>
+      </c>
+      <c r="C967" s="3" t="s">
+        <v>2742</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
directX rendering is basically functional
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BA3DEF5-3904-4E46-BB25-5824237A3D0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B31319E-0C4A-4B3B-8BCA-26903BD47817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4780" yWindow="160" windowWidth="24570" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2943" uniqueCount="2796">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2946" uniqueCount="2799">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -23651,6 +23651,16 @@
   <si>
     <t>仅在缩小时使用双线性插值缩放</t>
     <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Options.DirectXRendering</t>
+  </si>
+  <si>
+    <t>使用DirectX 11绘图</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Draw using DirectX 11</t>
   </si>
 </sst>
 </file>
@@ -24053,7 +24063,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D983"/>
+  <dimension ref="A1:D984"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -34868,6 +34878,17 @@
         <v>2793</v>
       </c>
     </row>
+    <row r="984" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A984" s="3" t="s">
+        <v>2796</v>
+      </c>
+      <c r="B984" s="4" t="s">
+        <v>2797</v>
+      </c>
+      <c r="C984" s="3" t="s">
+        <v>2798</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
support DesignatorRange and InhibitorRange
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B31319E-0C4A-4B3B-8BCA-26903BD47817}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0853A6F3-5326-4322-9439-EF7C04196A0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4780" yWindow="160" windowWidth="24570" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2946" uniqueCount="2799">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2952" uniqueCount="2805">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -23661,6 +23661,26 @@
   </si>
   <si>
     <t>Draw using DirectX 11</t>
+  </si>
+  <si>
+    <t>ViewDesignatorRangeInfo</t>
+  </si>
+  <si>
+    <t>ViewInhibitorRangeInfo</t>
+  </si>
+  <si>
+    <t>指示者范围</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>抑制者范围</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Designator Range</t>
+  </si>
+  <si>
+    <t>Inhibitor Range</t>
   </si>
 </sst>
 </file>
@@ -24063,7 +24083,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D984"/>
+  <dimension ref="A1:D986"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -34889,6 +34909,28 @@
         <v>2798</v>
       </c>
     </row>
+    <row r="985" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A985" s="3" t="s">
+        <v>2799</v>
+      </c>
+      <c r="B985" s="4" t="s">
+        <v>2801</v>
+      </c>
+      <c r="C985" s="3" t="s">
+        <v>2803</v>
+      </c>
+    </row>
+    <row r="986" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A986" s="3" t="s">
+        <v>2800</v>
+      </c>
+      <c r="B986" s="4" t="s">
+        <v>2802</v>
+      </c>
+      <c r="C986" s="3" t="s">
+        <v>2804</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix right click cancel & depth calcu for cliffs
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AB91445-8BC7-4D24-B1D8-E701294B965B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD610A29-C5D1-4DAF-9F6F-18B56E954BB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4780" yWindow="160" windowWidth="24570" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23656,13 +23656,6 @@
     <t>Options.DirectXRendering</t>
   </si>
   <si>
-    <t>使用DirectX 11绘图</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Draw using DirectX 11</t>
-  </si>
-  <si>
     <t>ViewDesignatorRangeInfo</t>
   </si>
   <si>
@@ -23691,6 +23684,13 @@
   </si>
   <si>
     <t>精确计算游戏对象间的深度关系（轻微影响性能）</t>
+  </si>
+  <si>
+    <t>使用 DirectX 11 (显卡) 绘图</t>
+  </si>
+  <si>
+    <t>Draw map using DirectX 11 (GPU)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -34913,43 +34913,43 @@
         <v>2796</v>
       </c>
       <c r="B984" s="4" t="s">
-        <v>2797</v>
+        <v>2806</v>
       </c>
       <c r="C984" s="3" t="s">
-        <v>2798</v>
+        <v>2807</v>
       </c>
     </row>
     <row r="985" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A985" s="3" t="s">
+        <v>2797</v>
+      </c>
+      <c r="B985" s="4" t="s">
         <v>2799</v>
       </c>
-      <c r="B985" s="4" t="s">
+      <c r="C985" s="3" t="s">
         <v>2801</v>
-      </c>
-      <c r="C985" s="3" t="s">
-        <v>2803</v>
       </c>
     </row>
     <row r="986" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A986" s="3" t="s">
+        <v>2798</v>
+      </c>
+      <c r="B986" s="4" t="s">
         <v>2800</v>
       </c>
-      <c r="B986" s="4" t="s">
+      <c r="C986" s="3" t="s">
         <v>2802</v>
-      </c>
-      <c r="C986" s="3" t="s">
-        <v>2804</v>
       </c>
     </row>
     <row r="987" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A987" s="3" t="s">
+        <v>2803</v>
+      </c>
+      <c r="B987" s="4" t="s">
         <v>2805</v>
       </c>
-      <c r="B987" s="4" t="s">
-        <v>2807</v>
-      </c>
       <c r="C987" s="3" t="s">
-        <v>2806</v>
+        <v>2804</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix shadow and object browser bug, add LoadObjectsOnInit
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD610A29-C5D1-4DAF-9F6F-18B56E954BB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29BED8C9-323D-474C-BCD6-F8BE4C47CB50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4780" yWindow="160" windowWidth="24570" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2955" uniqueCount="2808">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2961" uniqueCount="2814">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -23691,6 +23691,26 @@
   <si>
     <t>Draw map using DirectX 11 (GPU)</t>
     <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Loading objects, please wait...</t>
+  </si>
+  <si>
+    <t>InitAllObjectsProgressText</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Options.LoadObjectsOnInit</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Load all in-map objects during map initialization</t>
+  </si>
+  <si>
+    <t>加载单位中，请稍后...</t>
+  </si>
+  <si>
+    <t>在地图初始化时加载所有地图内对象</t>
   </si>
 </sst>
 </file>
@@ -24093,7 +24113,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D987"/>
+  <dimension ref="A1:D989"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -34952,6 +34972,28 @@
         <v>2804</v>
       </c>
     </row>
+    <row r="988" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A988" s="3" t="s">
+        <v>2809</v>
+      </c>
+      <c r="B988" s="4" t="s">
+        <v>2812</v>
+      </c>
+      <c r="C988" s="3" t="s">
+        <v>2808</v>
+      </c>
+    </row>
+    <row r="989" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A989" s="3" t="s">
+        <v>2810</v>
+      </c>
+      <c r="B989" s="4" t="s">
+        <v>2813</v>
+      </c>
+      <c r="C989" s="3" t="s">
+        <v>2811</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
trigger editor dropdown can display trigger disable info
rewrite house dialog
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29BED8C9-323D-474C-BCD6-F8BE4C47CB50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{849AF069-0AFF-4989-8D15-F548FF991162}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4780" yWindow="160" windowWidth="24570" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4830" yWindow="130" windowWidth="24570" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2961" uniqueCount="2814">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2979" uniqueCount="2830">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -23711,6 +23711,64 @@
   </si>
   <si>
     <t>在地图初始化时加载所有地图内对象</t>
+  </si>
+  <si>
+    <t>Please select parent country:</t>
+  </si>
+  <si>
+    <t>HousesRepairBaseNodes</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>HouseDialog.SelectParentCountry</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>选择继承国家：</t>
+  </si>
+  <si>
+    <t>维修基地节点 (Phobos B32+)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Repair BaseNodes (Phobos B32+)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Display whether triggers are disabled in the dropdown menu</t>
+  </si>
+  <si>
+    <t>在下拉菜单中显示触发是否被禁止</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Options.DisplayTriggerEnableInfo</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>HousesRepairBaseNodesMedium</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>简单</t>
+  </si>
+  <si>
+    <t>困难</t>
+  </si>
+  <si>
+    <t>普通</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>HousesRepairBaseNodesEasy</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>HousesRepairBaseNodesHard</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -24113,7 +24171,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D989"/>
+  <dimension ref="A1:D995"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -34994,6 +35052,72 @@
         <v>2811</v>
       </c>
     </row>
+    <row r="990" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A990" s="3" t="s">
+        <v>2816</v>
+      </c>
+      <c r="B990" s="4" t="s">
+        <v>2817</v>
+      </c>
+      <c r="C990" s="3" t="s">
+        <v>2814</v>
+      </c>
+    </row>
+    <row r="991" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A991" s="3" t="s">
+        <v>2815</v>
+      </c>
+      <c r="B991" s="4" t="s">
+        <v>2818</v>
+      </c>
+      <c r="C991" s="3" t="s">
+        <v>2819</v>
+      </c>
+    </row>
+    <row r="992" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A992" s="3" t="s">
+        <v>2822</v>
+      </c>
+      <c r="B992" s="4" t="s">
+        <v>2821</v>
+      </c>
+      <c r="C992" s="3" t="s">
+        <v>2820</v>
+      </c>
+    </row>
+    <row r="993" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A993" s="3" t="s">
+        <v>2827</v>
+      </c>
+      <c r="B993" s="4" t="s">
+        <v>2824</v>
+      </c>
+      <c r="C993" s="3" t="s">
+        <v>1221</v>
+      </c>
+    </row>
+    <row r="994" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A994" s="3" t="s">
+        <v>2823</v>
+      </c>
+      <c r="B994" s="4" t="s">
+        <v>2826</v>
+      </c>
+      <c r="C994" s="3" t="s">
+        <v>2828</v>
+      </c>
+    </row>
+    <row r="995" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A995" s="3" t="s">
+        <v>2829</v>
+      </c>
+      <c r="B995" s="4" t="s">
+        <v>2825</v>
+      </c>
+      <c r="C995" s="3" t="s">
+        <v>1223</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
search reference in trigger editor supports show params
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{849AF069-0AFF-4989-8D15-F548FF991162}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BD911FF-F0D8-47A4-A298-50DB8A5CE6C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4830" yWindow="130" windowWidth="24570" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2979" uniqueCount="2830">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2988" uniqueCount="2839">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -23768,6 +23768,38 @@
   </si>
   <si>
     <t>HousesRepairBaseNodesHard</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Param - Tag</t>
+  </si>
+  <si>
+    <t>Param - Team</t>
+  </si>
+  <si>
+    <t>Param - Trigger</t>
+  </si>
+  <si>
+    <t>SearhReference.TriggerParam.Tag</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SearhReference.TriggerParam.Team</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SearhReference.TriggerParam.Trigger</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>参数 - 标签</t>
+  </si>
+  <si>
+    <t>参数 - 小队</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>参数 - 触发</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -24171,7 +24203,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D995"/>
+  <dimension ref="A1:D998"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -35118,6 +35150,39 @@
         <v>1223</v>
       </c>
     </row>
+    <row r="996" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A996" s="3" t="s">
+        <v>2833</v>
+      </c>
+      <c r="B996" s="4" t="s">
+        <v>2836</v>
+      </c>
+      <c r="C996" s="3" t="s">
+        <v>2830</v>
+      </c>
+    </row>
+    <row r="997" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A997" s="3" t="s">
+        <v>2834</v>
+      </c>
+      <c r="B997" s="4" t="s">
+        <v>2837</v>
+      </c>
+      <c r="C997" s="3" t="s">
+        <v>2831</v>
+      </c>
+    </row>
+    <row r="998" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A998" s="3" t="s">
+        <v>2835</v>
+      </c>
+      <c r="B998" s="4" t="s">
+        <v>2838</v>
+      </c>
+      <c r="C998" s="3" t="s">
+        <v>2832</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
set directX rendering to default, add auto fallback
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7692DDFA-9142-40B8-8CEE-3E964D8E4AB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D15B135-4109-4A7E-97BF-EED3448B0DB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4830" yWindow="130" windowWidth="24570" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4850" yWindow="80" windowWidth="24570" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3000" uniqueCount="2851">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3003" uniqueCount="2854">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -23842,6 +23842,16 @@
   <si>
     <t>放置圆</t>
     <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>DirectXInitializationFailed</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Failed to initialize DirectX. Switching to DirectDraw rendering.</t>
+  </si>
+  <si>
+    <t>无法初始化DirectX，将切换至DirectDraw绘图。</t>
   </si>
 </sst>
 </file>
@@ -24244,7 +24254,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1002"/>
+  <dimension ref="A1:D1003"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -35268,6 +35278,17 @@
         <v>2842</v>
       </c>
     </row>
+    <row r="1003" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1003" s="3" t="s">
+        <v>2851</v>
+      </c>
+      <c r="B1003" s="4" t="s">
+        <v>2853</v>
+      </c>
+      <c r="C1003" s="3" t="s">
+        <v>2852</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
rewrite basic, singleplayer, special flag dialogs
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FCAA4D1-4CD1-4ED3-B2B4-B67B742BA791}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{090837AD-D8B6-4768-8C2C-EE460446507E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4850" yWindow="80" windowWidth="24570" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3012" uniqueCount="2863">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3080" uniqueCount="2931">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -23865,6 +23865,210 @@
   </si>
   <si>
     <t>Force Neutral and Special houses to use the light gray color in skirmish</t>
+  </si>
+  <si>
+    <t>SpecialFlags.Title</t>
+  </si>
+  <si>
+    <t>Special Flags</t>
+  </si>
+  <si>
+    <t>SpecialFlags.TiberiumGrows</t>
+  </si>
+  <si>
+    <t>Tiberium grows</t>
+  </si>
+  <si>
+    <t>SpecialFlags.TiberiumSpreads</t>
+  </si>
+  <si>
+    <t>Tiberium spreads</t>
+  </si>
+  <si>
+    <t>SpecialFlags.TiberiumExplosive</t>
+  </si>
+  <si>
+    <t>Tiberium explosive</t>
+  </si>
+  <si>
+    <t>SpecialFlags.DestroyableBridges</t>
+  </si>
+  <si>
+    <t>Destroyable bridges</t>
+  </si>
+  <si>
+    <t>SpecialFlags.MCVDeploy</t>
+  </si>
+  <si>
+    <t>MCV deploy</t>
+  </si>
+  <si>
+    <t>SpecialFlags.InitialVeteran</t>
+  </si>
+  <si>
+    <t>Initial veteran (initial troops have veteran status)</t>
+  </si>
+  <si>
+    <t>SpecialFlags.FixedAlliance</t>
+  </si>
+  <si>
+    <t>Fixed alliance</t>
+  </si>
+  <si>
+    <t>SpecialFlags.HarvesterImmune</t>
+  </si>
+  <si>
+    <t>Harvester immune</t>
+  </si>
+  <si>
+    <t>SpecialFlags.FogOfWar</t>
+  </si>
+  <si>
+    <t>Fog of war</t>
+  </si>
+  <si>
+    <t>SpecialFlags.Inert</t>
+  </si>
+  <si>
+    <t>Inert</t>
+  </si>
+  <si>
+    <t>SpecialFlags.IonStorms</t>
+  </si>
+  <si>
+    <t>Ion storms</t>
+  </si>
+  <si>
+    <t>SpecialFlags.Meteorites</t>
+  </si>
+  <si>
+    <t>Meteorites</t>
+  </si>
+  <si>
+    <t>SpecialFlags.Visceroids</t>
+  </si>
+  <si>
+    <t>Visceroids</t>
+  </si>
+  <si>
+    <t>SpecialFlags.Note</t>
+  </si>
+  <si>
+    <t>Note: some of the settings are probably just ignored</t>
+  </si>
+  <si>
+    <t>BasicHomeCell</t>
+  </si>
+  <si>
+    <t>Home Cell:</t>
+  </si>
+  <si>
+    <t>BasicAltHomeCell</t>
+  </si>
+  <si>
+    <t>Alt. Home Cell:</t>
+  </si>
+  <si>
+    <t>BasicRepairBaseNodes</t>
+  </si>
+  <si>
+    <t>Repair Base Nodes (Phobos B45+)</t>
+  </si>
+  <si>
+    <t>BasicMCVRedeploys</t>
+  </si>
+  <si>
+    <t>MCV Redeploys (Phobos B34+)</t>
+  </si>
+  <si>
+    <t>BasicShowBriefing</t>
+  </si>
+  <si>
+    <t>Show Briefing (Phobos B39+):</t>
+  </si>
+  <si>
+    <t>BasicBriefingTheme</t>
+  </si>
+  <si>
+    <t>Briefing Theme (Phobos B39+):</t>
+  </si>
+  <si>
+    <t>BasicTitle</t>
+  </si>
+  <si>
+    <t>Basic settings</t>
+  </si>
+  <si>
+    <t>Singleplayer Map Settings</t>
+  </si>
+  <si>
+    <t>特定标识</t>
+  </si>
+  <si>
+    <t>矿石生长</t>
+  </si>
+  <si>
+    <t>矿石蔓延</t>
+  </si>
+  <si>
+    <t>矿石爆炸(无效)</t>
+  </si>
+  <si>
+    <t>可摧毁桥梁(不影响C4/伊文)</t>
+  </si>
+  <si>
+    <t>基地车部署(无效)</t>
+  </si>
+  <si>
+    <t>初始精英(遭遇战初始单位精英)</t>
+  </si>
+  <si>
+    <t>固定联盟</t>
+  </si>
+  <si>
+    <t>矿车无敌(无效)</t>
+  </si>
+  <si>
+    <t>战争迷雾(半透明)</t>
+  </si>
+  <si>
+    <t>惰性效果</t>
+  </si>
+  <si>
+    <t>离子风暴(无效)</t>
+  </si>
+  <si>
+    <t>陨石(无效)</t>
+  </si>
+  <si>
+    <t>器官兽(无效)</t>
+  </si>
+  <si>
+    <t>一些设置只在特定情况下生效。</t>
+  </si>
+  <si>
+    <t>起始位置:</t>
+  </si>
+  <si>
+    <t>支线起始位置:</t>
+  </si>
+  <si>
+    <t>修复基地节点 (Phobos B45+)</t>
+  </si>
+  <si>
+    <t>允许基地车重新部署 (Phobos B34+)</t>
+  </si>
+  <si>
+    <t>显示任务简报 (Phobos B39+)</t>
+  </si>
+  <si>
+    <t>简报背景音乐 (Phobos B39+):</t>
+  </si>
+  <si>
+    <t>基本设置</t>
+  </si>
+  <si>
+    <t>单人任务设置</t>
   </si>
 </sst>
 </file>
@@ -24267,7 +24471,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1006"/>
+  <dimension ref="A1:D1029"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -35335,6 +35539,256 @@
         <v>2862</v>
       </c>
     </row>
+    <row r="1007" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1007" s="3" t="s">
+        <v>2863</v>
+      </c>
+      <c r="B1007" s="4" t="s">
+        <v>2908</v>
+      </c>
+      <c r="C1007" s="3" t="s">
+        <v>2864</v>
+      </c>
+    </row>
+    <row r="1008" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1008" s="3" t="s">
+        <v>2865</v>
+      </c>
+      <c r="B1008" s="4" t="s">
+        <v>2909</v>
+      </c>
+      <c r="C1008" s="3" t="s">
+        <v>2866</v>
+      </c>
+    </row>
+    <row r="1009" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1009" s="3" t="s">
+        <v>2867</v>
+      </c>
+      <c r="B1009" s="4" t="s">
+        <v>2910</v>
+      </c>
+      <c r="C1009" s="3" t="s">
+        <v>2868</v>
+      </c>
+    </row>
+    <row r="1010" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1010" s="3" t="s">
+        <v>2869</v>
+      </c>
+      <c r="B1010" s="4" t="s">
+        <v>2911</v>
+      </c>
+      <c r="C1010" s="3" t="s">
+        <v>2870</v>
+      </c>
+    </row>
+    <row r="1011" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1011" s="3" t="s">
+        <v>2871</v>
+      </c>
+      <c r="B1011" s="4" t="s">
+        <v>2912</v>
+      </c>
+      <c r="C1011" s="3" t="s">
+        <v>2872</v>
+      </c>
+    </row>
+    <row r="1012" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1012" s="3" t="s">
+        <v>2873</v>
+      </c>
+      <c r="B1012" s="4" t="s">
+        <v>2913</v>
+      </c>
+      <c r="C1012" s="3" t="s">
+        <v>2874</v>
+      </c>
+    </row>
+    <row r="1013" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1013" s="3" t="s">
+        <v>2875</v>
+      </c>
+      <c r="B1013" s="4" t="s">
+        <v>2914</v>
+      </c>
+      <c r="C1013" s="3" t="s">
+        <v>2876</v>
+      </c>
+    </row>
+    <row r="1014" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1014" s="3" t="s">
+        <v>2877</v>
+      </c>
+      <c r="B1014" s="4" t="s">
+        <v>2915</v>
+      </c>
+      <c r="C1014" s="3" t="s">
+        <v>2878</v>
+      </c>
+    </row>
+    <row r="1015" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1015" s="3" t="s">
+        <v>2879</v>
+      </c>
+      <c r="B1015" s="4" t="s">
+        <v>2916</v>
+      </c>
+      <c r="C1015" s="3" t="s">
+        <v>2880</v>
+      </c>
+    </row>
+    <row r="1016" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1016" s="3" t="s">
+        <v>2881</v>
+      </c>
+      <c r="B1016" s="4" t="s">
+        <v>2917</v>
+      </c>
+      <c r="C1016" s="3" t="s">
+        <v>2882</v>
+      </c>
+    </row>
+    <row r="1017" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1017" s="3" t="s">
+        <v>2883</v>
+      </c>
+      <c r="B1017" s="4" t="s">
+        <v>2918</v>
+      </c>
+      <c r="C1017" s="3" t="s">
+        <v>2884</v>
+      </c>
+    </row>
+    <row r="1018" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1018" s="3" t="s">
+        <v>2885</v>
+      </c>
+      <c r="B1018" s="4" t="s">
+        <v>2919</v>
+      </c>
+      <c r="C1018" s="3" t="s">
+        <v>2886</v>
+      </c>
+    </row>
+    <row r="1019" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1019" s="3" t="s">
+        <v>2887</v>
+      </c>
+      <c r="B1019" s="4" t="s">
+        <v>2920</v>
+      </c>
+      <c r="C1019" s="3" t="s">
+        <v>2888</v>
+      </c>
+    </row>
+    <row r="1020" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1020" s="3" t="s">
+        <v>2889</v>
+      </c>
+      <c r="B1020" s="4" t="s">
+        <v>2921</v>
+      </c>
+      <c r="C1020" s="3" t="s">
+        <v>2890</v>
+      </c>
+    </row>
+    <row r="1021" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1021" s="3" t="s">
+        <v>2891</v>
+      </c>
+      <c r="B1021" s="4" t="s">
+        <v>2922</v>
+      </c>
+      <c r="C1021" s="3" t="s">
+        <v>2892</v>
+      </c>
+    </row>
+    <row r="1022" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1022" s="3" t="s">
+        <v>2893</v>
+      </c>
+      <c r="B1022" s="4" t="s">
+        <v>2923</v>
+      </c>
+      <c r="C1022" s="3" t="s">
+        <v>2894</v>
+      </c>
+    </row>
+    <row r="1023" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1023" s="3" t="s">
+        <v>2895</v>
+      </c>
+      <c r="B1023" s="4" t="s">
+        <v>2924</v>
+      </c>
+      <c r="C1023" s="3" t="s">
+        <v>2896</v>
+      </c>
+    </row>
+    <row r="1024" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1024" s="3" t="s">
+        <v>2897</v>
+      </c>
+      <c r="B1024" s="4" t="s">
+        <v>2925</v>
+      </c>
+      <c r="C1024" s="3" t="s">
+        <v>2898</v>
+      </c>
+    </row>
+    <row r="1025" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1025" s="3" t="s">
+        <v>2899</v>
+      </c>
+      <c r="B1025" s="4" t="s">
+        <v>2926</v>
+      </c>
+      <c r="C1025" s="3" t="s">
+        <v>2900</v>
+      </c>
+    </row>
+    <row r="1026" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1026" s="3" t="s">
+        <v>2901</v>
+      </c>
+      <c r="B1026" s="4" t="s">
+        <v>2927</v>
+      </c>
+      <c r="C1026" s="3" t="s">
+        <v>2902</v>
+      </c>
+    </row>
+    <row r="1027" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1027" s="3" t="s">
+        <v>2903</v>
+      </c>
+      <c r="B1027" s="4" t="s">
+        <v>2928</v>
+      </c>
+      <c r="C1027" s="3" t="s">
+        <v>2904</v>
+      </c>
+    </row>
+    <row r="1028" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1028" s="3" t="s">
+        <v>2905</v>
+      </c>
+      <c r="B1028" s="4" t="s">
+        <v>2929</v>
+      </c>
+      <c r="C1028" s="3" t="s">
+        <v>2906</v>
+      </c>
+    </row>
+    <row r="1029" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B1029" s="4" t="s">
+        <v>2930</v>
+      </c>
+      <c r="C1029" s="3" t="s">
+        <v>2907</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
search reference can search tag attached objects
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{090837AD-D8B6-4768-8C2C-EE460446507E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72882206-FD5E-4991-B6B5-F38ECBBE5D91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4850" yWindow="80" windowWidth="24570" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3080" uniqueCount="2931">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3087" uniqueCount="2937">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -24069,6 +24069,27 @@
   </si>
   <si>
     <t>单人任务设置</t>
+  </si>
+  <si>
+    <t>SingleplayerTitle</t>
+  </si>
+  <si>
+    <t>SearhReference.TagObject</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Object</t>
+  </si>
+  <si>
+    <t>对象</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SearhReference.TagTag</t>
+  </si>
+  <si>
+    <t>Tag</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -24471,7 +24492,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1029"/>
+  <dimension ref="A1:D1031"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -35782,11 +35803,36 @@
       </c>
     </row>
     <row r="1029" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1029" s="3" t="s">
+        <v>2931</v>
+      </c>
       <c r="B1029" s="4" t="s">
         <v>2930</v>
       </c>
       <c r="C1029" s="3" t="s">
         <v>2907</v>
+      </c>
+    </row>
+    <row r="1030" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1030" s="3" t="s">
+        <v>2932</v>
+      </c>
+      <c r="B1030" s="4" t="s">
+        <v>2934</v>
+      </c>
+      <c r="C1030" s="3" t="s">
+        <v>2933</v>
+      </c>
+    </row>
+    <row r="1031" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1031" s="3" t="s">
+        <v>2935</v>
+      </c>
+      <c r="B1031" s="4" t="s">
+        <v>1752</v>
+      </c>
+      <c r="C1031" s="3" t="s">
+        <v>2936</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add follow active window button
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE45B8C9-551D-4531-8B08-E523FC661A9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{095B1BC6-BA67-4814-B783-DDA7C4D930D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4600" yWindow="550" windowWidth="28900" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3090" uniqueCount="2940">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3096" uniqueCount="2946">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -24099,6 +24099,26 @@
   </si>
   <si>
     <t>紧凑排列地形浏览器的图像</t>
+  </si>
+  <si>
+    <t>SearhReference.AttachedTrigger</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Attached Trigger</t>
+  </si>
+  <si>
+    <t>关联触发</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SearchReferenceFollowActiveWindow</t>
+  </si>
+  <si>
+    <t>Follow active window</t>
+  </si>
+  <si>
+    <t>跟随活动窗口</t>
   </si>
 </sst>
 </file>
@@ -24501,7 +24521,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1032"/>
+  <dimension ref="A1:D1034"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -35855,6 +35875,28 @@
         <v>2937</v>
       </c>
     </row>
+    <row r="1033" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1033" s="3" t="s">
+        <v>2940</v>
+      </c>
+      <c r="B1033" s="4" t="s">
+        <v>2942</v>
+      </c>
+      <c r="C1033" s="3" t="s">
+        <v>2941</v>
+      </c>
+    </row>
+    <row r="1034" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1034" s="3" t="s">
+        <v>2943</v>
+      </c>
+      <c r="B1034" s="4" t="s">
+        <v>2945</v>
+      </c>
+      <c r="C1034" s="3" t="s">
+        <v>2944</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
mouse commands can record brush size
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{095B1BC6-BA67-4814-B783-DDA7C4D930D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{036CF52E-147E-49E3-A58C-94CF4C8631E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4600" yWindow="550" windowWidth="28900" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3096" uniqueCount="2946">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3099" uniqueCount="2949">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -24119,6 +24119,16 @@
   </si>
   <si>
     <t>跟随活动窗口</t>
+  </si>
+  <si>
+    <t>Options.RecordBrushSizeHistory</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>记忆各操作的笔刷大小</t>
+  </si>
+  <si>
+    <t>Remember brush sizes for mouse commands</t>
   </si>
 </sst>
 </file>
@@ -24521,7 +24531,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1034"/>
+  <dimension ref="A1:D1035"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -35897,6 +35907,17 @@
         <v>2944</v>
       </c>
     </row>
+    <row r="1035" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1035" s="3" t="s">
+        <v>2946</v>
+      </c>
+      <c r="B1035" s="4" t="s">
+        <v>2947</v>
+      </c>
+      <c r="C1035" s="3" t="s">
+        <v>2948</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
multi sel can show different ore values, improve scaling performance
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{036CF52E-147E-49E3-A58C-94CF4C8631E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8551E0D5-0D48-45F7-BF19-7E1C5DBF5343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4600" yWindow="550" windowWidth="28900" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3099" uniqueCount="2949">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3111" uniqueCount="2961">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -24129,6 +24129,46 @@
   </si>
   <si>
     <t>Remember brush sizes for mouse commands</t>
+  </si>
+  <si>
+    <t>MoneyOnMap.MultiSelection.Riparius</t>
+  </si>
+  <si>
+    <t>MoneyOnMap.MultiSelection.Cruentus</t>
+  </si>
+  <si>
+    <t>MoneyOnMap.MultiSelection.Vinifera</t>
+  </si>
+  <si>
+    <t>MoneyOnMap.MultiSelection.Aboreus</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>, 金矿: %d</t>
+  </si>
+  <si>
+    <t>, 水晶: %d</t>
+  </si>
+  <si>
+    <t>, 矿石3: %d</t>
+  </si>
+  <si>
+    <t>, 矿石4: %d</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>, Ore: %d</t>
+  </si>
+  <si>
+    <t>, Gems: %d</t>
+  </si>
+  <si>
+    <t>, Ore 3: %d</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>, Ore 4: %d</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -24531,7 +24571,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1035"/>
+  <dimension ref="A1:D1039"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -35918,6 +35958,50 @@
         <v>2948</v>
       </c>
     </row>
+    <row r="1036" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1036" s="3" t="s">
+        <v>2949</v>
+      </c>
+      <c r="B1036" s="4" t="s">
+        <v>2953</v>
+      </c>
+      <c r="C1036" s="3" t="s">
+        <v>2957</v>
+      </c>
+    </row>
+    <row r="1037" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1037" s="3" t="s">
+        <v>2950</v>
+      </c>
+      <c r="B1037" s="4" t="s">
+        <v>2954</v>
+      </c>
+      <c r="C1037" s="3" t="s">
+        <v>2958</v>
+      </c>
+    </row>
+    <row r="1038" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1038" s="3" t="s">
+        <v>2951</v>
+      </c>
+      <c r="B1038" s="4" t="s">
+        <v>2955</v>
+      </c>
+      <c r="C1038" s="3" t="s">
+        <v>2959</v>
+      </c>
+    </row>
+    <row r="1039" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1039" s="3" t="s">
+        <v>2952</v>
+      </c>
+      <c r="B1039" s="4" t="s">
+        <v>2956</v>
+      </c>
+      <c r="C1039" s="3" t="s">
+        <v>2960</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add new lua scripts, add theme options, implement random tree dlg for mirage disguise
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6C20FC5-0993-4901-887D-BC8976C02360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A380B3C0-3BB4-4831-A2FD-5DAB15306D8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4600" yWindow="550" windowWidth="28900" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3114" uniqueCount="2964">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3132" uniqueCount="2982">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -24165,6 +24165,68 @@
   </si>
   <si>
     <t>TriggerNewShort</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>BasicTheme</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>背景音乐:</t>
+  </si>
+  <si>
+    <t>BasicLoadingTheme</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>加载界面背景音乐 (Ares 0.7+):</t>
+  </si>
+  <si>
+    <t>Theme:</t>
+  </si>
+  <si>
+    <t>Loading Theme (Ares 0.7+):</t>
+  </si>
+  <si>
+    <t>RandomTreeDisguiseDesc</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Set mirage disguise trees</t>
+  </si>
+  <si>
+    <t>RandomTreeDisguiseTitle</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Mirage disguise trees</t>
+  </si>
+  <si>
+    <t>选择幻影伪装的树木</t>
+  </si>
+  <si>
+    <t>幻影伪装树木</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>RandomTreeTitle</t>
+  </si>
+  <si>
+    <t>RandomTreeDesc</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>请选择准备放置的树木</t>
+  </si>
+  <si>
+    <t>绘制随机树木</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Please select the trees that shall be placed</t>
+  </si>
+  <si>
+    <t>Random Tree Placing</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -24568,7 +24630,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1040"/>
+  <dimension ref="A1:D1046"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -36010,6 +36072,72 @@
         <v>2959</v>
       </c>
     </row>
+    <row r="1041" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1041" s="3" t="s">
+        <v>2964</v>
+      </c>
+      <c r="B1041" s="4" t="s">
+        <v>2965</v>
+      </c>
+      <c r="C1041" s="3" t="s">
+        <v>2968</v>
+      </c>
+    </row>
+    <row r="1042" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1042" s="3" t="s">
+        <v>2966</v>
+      </c>
+      <c r="B1042" s="4" t="s">
+        <v>2967</v>
+      </c>
+      <c r="C1042" s="3" t="s">
+        <v>2969</v>
+      </c>
+    </row>
+    <row r="1043" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1043" s="3" t="s">
+        <v>2970</v>
+      </c>
+      <c r="B1043" s="4" t="s">
+        <v>2974</v>
+      </c>
+      <c r="C1043" s="3" t="s">
+        <v>2971</v>
+      </c>
+    </row>
+    <row r="1044" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1044" s="3" t="s">
+        <v>2972</v>
+      </c>
+      <c r="B1044" s="4" t="s">
+        <v>2975</v>
+      </c>
+      <c r="C1044" s="3" t="s">
+        <v>2973</v>
+      </c>
+    </row>
+    <row r="1045" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1045" s="3" t="s">
+        <v>2976</v>
+      </c>
+      <c r="B1045" s="4" t="s">
+        <v>2979</v>
+      </c>
+      <c r="C1045" s="3" t="s">
+        <v>2981</v>
+      </c>
+    </row>
+    <row r="1046" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1046" s="3" t="s">
+        <v>2977</v>
+      </c>
+      <c r="B1046" s="4" t="s">
+        <v>2978</v>
+      </c>
+      <c r="C1046" s="3" t="s">
+        <v>2980</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add floating tile browser
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F555862-A8E0-4BEF-A41D-B5095E92DB7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{760232C2-597E-4569-B7A5-C9107E39DBF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3147" uniqueCount="2997">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3150" uniqueCount="3000">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -24278,6 +24278,16 @@
   </si>
   <si>
     <t>禁用Lua脚本安全检查</t>
+  </si>
+  <si>
+    <t>Options.TileSetBrowserFloating</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>将地形浏览器作为独立窗口显示</t>
+  </si>
+  <si>
+    <t>Tile browser as floating window</t>
   </si>
 </sst>
 </file>
@@ -24680,7 +24690,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1051"/>
+  <dimension ref="A1:D1052"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -36243,6 +36253,17 @@
         <v>2995</v>
       </c>
     </row>
+    <row r="1052" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1052" s="3" t="s">
+        <v>2997</v>
+      </c>
+      <c r="B1052" s="4" t="s">
+        <v>2998</v>
+      </c>
+      <c r="C1052" s="3" t="s">
+        <v>2999</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add floating view object
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{760232C2-597E-4569-B7A5-C9107E39DBF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E7A2D7E-4F79-4374-9AD7-98A9E9388006}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3150" uniqueCount="3000">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3153" uniqueCount="3003">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -24288,6 +24288,16 @@
   </si>
   <si>
     <t>Tile browser as floating window</t>
+  </si>
+  <si>
+    <t>Options.ViewObjectsFloating</t>
+  </si>
+  <si>
+    <t>Object browser as floating window</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>将物品浏览器作为独立窗口显示</t>
   </si>
 </sst>
 </file>
@@ -24690,7 +24700,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1052"/>
+  <dimension ref="A1:D1053"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -36264,6 +36274,17 @@
         <v>2999</v>
       </c>
     </row>
+    <row r="1053" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1053" s="3" t="s">
+        <v>3000</v>
+      </c>
+      <c r="B1053" s="4" t="s">
+        <v>3002</v>
+      </c>
+      <c r="C1053" s="3" t="s">
+        <v>3001</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add two toolbar buttons
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{148763F4-196A-481F-881A-9A09FB568B72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAC64607-B989-4976-A10B-79D51F6CAE7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3165" uniqueCount="3015">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3168" uniqueCount="3018">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -24336,6 +24336,18 @@
   </si>
   <si>
     <t>Opaque (100%)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>全透明(1%)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>1% Opacity</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>TransparencyMenu.1</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -24739,7 +24751,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1057"/>
+  <dimension ref="A1:D1058"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -36368,6 +36380,17 @@
         <v>3013</v>
       </c>
     </row>
+    <row r="1058" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1058" s="3" t="s">
+        <v>3017</v>
+      </c>
+      <c r="B1058" s="4" t="s">
+        <v>3015</v>
+      </c>
+      <c r="C1058" s="3" t="s">
+        <v>3016</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
change vertex mode cursor, fix ellipse border bug
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{654124E5-06C4-48C9-BFDF-EEE43CDCBD04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A67810AE-26E7-4EC5-8851-9A88A1B28213}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="490" windowWidth="28900" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24200,18 +24200,10 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>Shift: Steep slope, Ctrl+Shift:  Ignore non-morphable tiles, A: Switch vertex mode, Up/Down: Raise/lower tile</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>Ctrl: 抬升/降低同类地表（非顶点模式），Shift: 陡峭斜面，Ctrl+Shift: 无视不可抬升/降低地形，A：切换顶点模式</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>Shift: 陡峭斜面，Ctrl+Shift: 无视不可抬升/降低地形，A：切换顶点模式，Up/Down：抬升或降低地表</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>VertexModeOn</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -24237,6 +24229,14 @@
   </si>
   <si>
     <t>Zoom: %.02fx, middle-click to reset</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Shift: 陡峭斜面，Ctrl+Shift: 无视不可抬升/降低地形，A：切换顶点模式，Up/Down/滚轮：抬升或降低地表</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Shift: Steep slope, Ctrl+Shift:  Ignore non-morphable tiles, A: Switch vertex mode, Up/Down/Mouse wheel: Raise/lower tile</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -25981,7 +25981,7 @@
         <v>116</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>3015</v>
+        <v>3014</v>
       </c>
       <c r="C123" s="3" t="s">
         <v>3013</v>
@@ -25992,10 +25992,10 @@
         <v>117</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>3016</v>
+        <v>3022</v>
       </c>
       <c r="C124" s="3" t="s">
-        <v>3014</v>
+        <v>3023</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.4">
@@ -32977,7 +32977,7 @@
         <v>2570</v>
       </c>
       <c r="C759" s="3" t="s">
-        <v>3023</v>
+        <v>3021</v>
       </c>
     </row>
     <row r="760" spans="1:3" x14ac:dyDescent="0.4">
@@ -36282,24 +36282,24 @@
     </row>
     <row r="1059" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1059" s="3" t="s">
+        <v>3015</v>
+      </c>
+      <c r="B1059" s="4" t="s">
+        <v>3016</v>
+      </c>
+      <c r="C1059" s="3" t="s">
         <v>3017</v>
-      </c>
-      <c r="B1059" s="4" t="s">
-        <v>3018</v>
-      </c>
-      <c r="C1059" s="3" t="s">
-        <v>3019</v>
       </c>
     </row>
     <row r="1060" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1060" s="3" t="s">
+        <v>3018</v>
+      </c>
+      <c r="B1060" s="4" t="s">
+        <v>3019</v>
+      </c>
+      <c r="C1060" s="3" t="s">
         <v>3020</v>
-      </c>
-      <c r="B1060" s="4" t="s">
-        <v>3021</v>
-      </c>
-      <c r="C1060" s="3" t="s">
-        <v>3022</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add option to reload game ini when opening map
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBCCEA2E-60F4-4C5E-8710-32289E6292A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CEC31C2-FEAD-4818-8405-3C87E0CAF4AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="490" windowWidth="28900" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3168" uniqueCount="3017">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3171" uniqueCount="3020">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -24049,6 +24049,15 @@
   </si>
   <si>
     <t>避让不可抬升地形</t>
+  </si>
+  <si>
+    <t>Options.ReloadIniWhenOpeningMap</t>
+  </si>
+  <si>
+    <t>Reload game INIs when opening map file</t>
+  </si>
+  <si>
+    <t>打开地图时重新加载游戏ini</t>
   </si>
 </sst>
 </file>
@@ -24451,7 +24460,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1058"/>
+  <dimension ref="A1:D1059"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -36091,6 +36100,17 @@
         <v>3015</v>
       </c>
     </row>
+    <row r="1059" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1059" s="3" t="s">
+        <v>3017</v>
+      </c>
+      <c r="B1059" s="4" t="s">
+        <v>3019</v>
+      </c>
+      <c r="C1059" s="3" t="s">
+        <v>3018</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add confirm dialog in reload map
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CEC31C2-FEAD-4818-8405-3C87E0CAF4AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9731764A-2BE7-4C1F-B37E-B5D422BD4393}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="490" windowWidth="28900" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3171" uniqueCount="3020">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3177" uniqueCount="3026">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -24058,6 +24058,26 @@
   </si>
   <si>
     <t>打开地图时重新加载游戏ini</t>
+  </si>
+  <si>
+    <t>ReloadMapConfirmTitle</t>
+  </si>
+  <si>
+    <t>ReloadMapConfirmMessage</t>
+  </si>
+  <si>
+    <t>Reload Map Confirm</t>
+  </si>
+  <si>
+    <t>Are you sure you want to reload the map?</t>
+  </si>
+  <si>
+    <t>重载地图确认</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>确认要重新加载地图吗？</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -24460,7 +24480,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1059"/>
+  <dimension ref="A1:D1061"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -36111,6 +36131,28 @@
         <v>3018</v>
       </c>
     </row>
+    <row r="1060" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1060" s="3" t="s">
+        <v>3020</v>
+      </c>
+      <c r="B1060" s="4" t="s">
+        <v>3024</v>
+      </c>
+      <c r="C1060" s="3" t="s">
+        <v>3022</v>
+      </c>
+    </row>
+    <row r="1061" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1061" s="3" t="s">
+        <v>3021</v>
+      </c>
+      <c r="B1061" s="4" t="s">
+        <v>3025</v>
+      </c>
+      <c r="C1061" s="3" t="s">
+        <v>3023</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
support SetRecruitableOnLiberate & <Alternate Next Scenario>
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCAF02AA-55C0-40BB-80C1-060BC4BB9283}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53053490-3FF0-465F-B240-510F7DBF2BD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5120" yWindow="2710" windowWidth="28900" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1160" yWindow="1460" windowWidth="28900" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3273" uniqueCount="3112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3291" uniqueCount="3130">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -24316,6 +24316,67 @@
   <si>
     <t>生命值 (%)</t>
     <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>不使用本逻辑</t>
+  </si>
+  <si>
+    <t>设为不可重组</t>
+  </si>
+  <si>
+    <t>设为可重组</t>
+  </si>
+  <si>
+    <t>SetRecruitOnLiber.1</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SetRecruitOnLiber.0</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SetRecruitOnLiber.-1</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>解散重组:</t>
+  </si>
+  <si>
+    <t>TeamTypesTooltipSetRecruitOnLiber</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>TeamTypesLabelSetRecruitOnLiber</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>(Phobos v0.5-alpha+) 在原版游戏中，当单位被加入到小队中时，其 RecruitableB 字段会被小队的设置 AreTeamMembersRecruitable 覆写。单位被小队释放时，该字段也不会被恢复。本设置允许小队在释放时重新设置该字段。默认为 [General]-&gt;SetRecruitableOnLiberate。</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Don't use this logic</t>
+  </si>
+  <si>
+    <t>Marked as not recruitable</t>
+  </si>
+  <si>
+    <t>Marked as recruitable</t>
+  </si>
+  <si>
+    <t>Rec/Lib:</t>
+  </si>
+  <si>
+    <t>Phobos v0.5-alpha+) In vanilla, when a unit is added to a team, its RecruitableB flag is overwritten by the team's AreTeamMembersRecruitable setting. When the unit is liberated from the team, the flag is not restored. This setting allows a team to reset this flag when liberating its members. Default [General]-&gt;SetRecruitableOnLiberate.</t>
+  </si>
+  <si>
+    <t>LocalVariablesAltTooltip</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>(Phobos v0.5-alpha+) Using [Basic]-&gt;SkipMapSelect=yes in the map file allows you to bypass the restriction in mapselmd.ini-which requires that the player's faction in the current campaign must match the faction in the next new campaign.\nYou can use NextScenario and AltNextScenario to specify the map names required to enter a new campaign, thereby forcing the game to proceed to the next campaign.\nSetting a local variable named &lt;Alternate Next Scenario&gt; will also trigger AltNextScenario.</t>
+  </si>
+  <si>
+    <t>(Phobos v0.5-alpha+) 在地图文件中使用 [Basic]-&gt;SkipMapSelect=yes （跳过地图选择）可以绕过 mapselmd.ini中的限制——该限制要求当前战役中玩家所属的阵营必须与下一个新战役中的阵营一致。\n你可以使用 NextScenari（下一主线剧情）和 AltNextScenario （下一支线剧情）来指定进入新战役所需的地图名称强制游戏进入下一个战役。\n启用一个名为 &lt;Alternate Next Scenario&gt; 的局部变量也可以触发 AltNextScenario。</t>
   </si>
 </sst>
 </file>
@@ -24733,7 +24794,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1093"/>
+  <dimension ref="A1:D1099"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -36758,6 +36819,72 @@
         <v>3109</v>
       </c>
     </row>
+    <row r="1094" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1094" s="3" t="s">
+        <v>3117</v>
+      </c>
+      <c r="B1094" s="4" t="s">
+        <v>3112</v>
+      </c>
+      <c r="C1094" s="3" t="s">
+        <v>3122</v>
+      </c>
+    </row>
+    <row r="1095" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1095" s="3" t="s">
+        <v>3116</v>
+      </c>
+      <c r="B1095" s="4" t="s">
+        <v>3113</v>
+      </c>
+      <c r="C1095" s="3" t="s">
+        <v>3123</v>
+      </c>
+    </row>
+    <row r="1096" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1096" s="3" t="s">
+        <v>3115</v>
+      </c>
+      <c r="B1096" s="4" t="s">
+        <v>3114</v>
+      </c>
+      <c r="C1096" s="3" t="s">
+        <v>3124</v>
+      </c>
+    </row>
+    <row r="1097" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1097" s="3" t="s">
+        <v>3120</v>
+      </c>
+      <c r="B1097" s="4" t="s">
+        <v>3118</v>
+      </c>
+      <c r="C1097" s="3" t="s">
+        <v>3125</v>
+      </c>
+    </row>
+    <row r="1098" spans="1:3" ht="112" x14ac:dyDescent="0.4">
+      <c r="A1098" s="3" t="s">
+        <v>3119</v>
+      </c>
+      <c r="B1098" s="4" t="s">
+        <v>3121</v>
+      </c>
+      <c r="C1098" s="3" t="s">
+        <v>3126</v>
+      </c>
+    </row>
+    <row r="1099" spans="1:3" ht="152" x14ac:dyDescent="0.4">
+      <c r="A1099" s="3" t="s">
+        <v>3127</v>
+      </c>
+      <c r="B1099" s="4" t="s">
+        <v>3129</v>
+      </c>
+      <c r="C1099" s="3" t="s">
+        <v>3128</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
add path finding distance tool
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53053490-3FF0-465F-B240-510F7DBF2BD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F1FAFCD-3D14-4A99-B6D3-029D35D01E9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1160" yWindow="1460" windowWidth="28900" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3291" uniqueCount="3130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3327" uniqueCount="3165">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -24377,6 +24377,126 @@
   </si>
   <si>
     <t>(Phobos v0.5-alpha+) 在地图文件中使用 [Basic]-&gt;SkipMapSelect=yes （跳过地图选择）可以绕过 mapselmd.ini中的限制——该限制要求当前战役中玩家所属的阵营必须与下一个新战役中的阵营一致。\n你可以使用 NextScenari（下一主线剧情）和 AltNextScenario （下一支线剧情）来指定进入新战役所需的地图名称强制游戏进入下一个战役。\n启用一个名为 &lt;Alternate Next Scenario&gt; 的局部变量也可以触发 AltNextScenario。</t>
+  </si>
+  <si>
+    <t>寻路距离</t>
+  </si>
+  <si>
+    <t>寻路测距</t>
+  </si>
+  <si>
+    <t>寻路类型:</t>
+  </si>
+  <si>
+    <t>MeasurementToolbox.MovementZone</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MeasurementToolbox.PathDistanceGroup</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MeasurementToolbox.PathDistance</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MeasurementToolbox.DestructibleOverlay</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MeasurementToolbox.DestructibleUnits</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>可摧毁\n单位</t>
+  </si>
+  <si>
+    <t>可摧毁\n覆盖物</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MeasurementToolbox.ClearPathDistance</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>清除路径</t>
+  </si>
+  <si>
+    <t>MeasurementToolbox.PathType.NormalLand</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MeasurementToolbox.PathType.NormalSea</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MeasurementToolbox.PathType.NormalAmphibian</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>陆地</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>海面</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>两栖</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>火车</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MeasurementToolbox.PathType.Train</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Path Distance</t>
+  </si>
+  <si>
+    <t>MovementZone:</t>
+  </si>
+  <si>
+    <t>Destructible\nOverlay</t>
+  </si>
+  <si>
+    <t>Destructible\nUnits</t>
+  </si>
+  <si>
+    <t>Clear Paths</t>
+  </si>
+  <si>
+    <t>Land</t>
+  </si>
+  <si>
+    <t>Sea</t>
+  </si>
+  <si>
+    <t>Amphibian</t>
+  </si>
+  <si>
+    <t>Train</t>
+  </si>
+  <si>
+    <t>DistanceRuler.PathDistance</t>
+  </si>
+  <si>
+    <t>DistanceRuler.PathUnreachable</t>
+  </si>
+  <si>
+    <t>寻路距离: %s</t>
+  </si>
+  <si>
+    <t>寻路距离: 无法到达</t>
+  </si>
+  <si>
+    <t>Path Distance: %s</t>
+  </si>
+  <si>
+    <t>Path Distance: Unreachable</t>
   </si>
 </sst>
 </file>
@@ -24794,7 +24914,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1099"/>
+  <dimension ref="A1:D1111"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -36863,7 +36983,7 @@
         <v>3125</v>
       </c>
     </row>
-    <row r="1098" spans="1:3" ht="112" x14ac:dyDescent="0.4">
+    <row r="1098" spans="1:3" ht="114" x14ac:dyDescent="0.4">
       <c r="A1098" s="3" t="s">
         <v>3119</v>
       </c>
@@ -36883,6 +37003,138 @@
       </c>
       <c r="C1099" s="3" t="s">
         <v>3128</v>
+      </c>
+    </row>
+    <row r="1100" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1100" s="3" t="s">
+        <v>3135</v>
+      </c>
+      <c r="B1100" s="4" t="s">
+        <v>3130</v>
+      </c>
+      <c r="C1100" s="3" t="s">
+        <v>3150</v>
+      </c>
+    </row>
+    <row r="1101" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1101" s="3" t="s">
+        <v>3134</v>
+      </c>
+      <c r="B1101" s="4" t="s">
+        <v>3131</v>
+      </c>
+      <c r="C1101" s="3" t="s">
+        <v>3150</v>
+      </c>
+    </row>
+    <row r="1102" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1102" s="3" t="s">
+        <v>3133</v>
+      </c>
+      <c r="B1102" s="4" t="s">
+        <v>3132</v>
+      </c>
+      <c r="C1102" s="3" t="s">
+        <v>3151</v>
+      </c>
+    </row>
+    <row r="1103" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1103" s="3" t="s">
+        <v>3136</v>
+      </c>
+      <c r="B1103" s="4" t="s">
+        <v>3139</v>
+      </c>
+      <c r="C1103" s="3" t="s">
+        <v>3152</v>
+      </c>
+    </row>
+    <row r="1104" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1104" s="3" t="s">
+        <v>3137</v>
+      </c>
+      <c r="B1104" s="4" t="s">
+        <v>3138</v>
+      </c>
+      <c r="C1104" s="3" t="s">
+        <v>3153</v>
+      </c>
+    </row>
+    <row r="1105" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1105" s="3" t="s">
+        <v>3140</v>
+      </c>
+      <c r="B1105" s="4" t="s">
+        <v>3141</v>
+      </c>
+      <c r="C1105" s="3" t="s">
+        <v>3154</v>
+      </c>
+    </row>
+    <row r="1106" spans="1:3" ht="38" x14ac:dyDescent="0.4">
+      <c r="A1106" s="3" t="s">
+        <v>3142</v>
+      </c>
+      <c r="B1106" s="4" t="s">
+        <v>3145</v>
+      </c>
+      <c r="C1106" s="3" t="s">
+        <v>3155</v>
+      </c>
+    </row>
+    <row r="1107" spans="1:3" ht="38" x14ac:dyDescent="0.4">
+      <c r="A1107" s="3" t="s">
+        <v>3143</v>
+      </c>
+      <c r="B1107" s="4" t="s">
+        <v>3146</v>
+      </c>
+      <c r="C1107" s="3" t="s">
+        <v>3156</v>
+      </c>
+    </row>
+    <row r="1108" spans="1:3" ht="38" x14ac:dyDescent="0.4">
+      <c r="A1108" s="3" t="s">
+        <v>3144</v>
+      </c>
+      <c r="B1108" s="4" t="s">
+        <v>3147</v>
+      </c>
+      <c r="C1108" s="3" t="s">
+        <v>3157</v>
+      </c>
+    </row>
+    <row r="1109" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1109" s="3" t="s">
+        <v>3149</v>
+      </c>
+      <c r="B1109" s="4" t="s">
+        <v>3148</v>
+      </c>
+      <c r="C1109" s="3" t="s">
+        <v>3158</v>
+      </c>
+    </row>
+    <row r="1110" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1110" s="3" t="s">
+        <v>3159</v>
+      </c>
+      <c r="B1110" s="4" t="s">
+        <v>3161</v>
+      </c>
+      <c r="C1110" s="3" t="s">
+        <v>3163</v>
+      </c>
+    </row>
+    <row r="1111" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1111" s="3" t="s">
+        <v>3160</v>
+      </c>
+      <c r="B1111" s="4" t="s">
+        <v>3162</v>
+      </c>
+      <c r="C1111" s="3" t="s">
+        <v>3164</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add autoconnect feature to PlaceConnectedTile
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED9DD319-6313-4056-9D66-DFFD9FF4ADF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4A23FD4-2FBF-4A21-8DAC-E1585B94044A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13130" yWindow="580" windowWidth="28900" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3020" yWindow="760" windowWidth="28900" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3354" uniqueCount="3192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3360" uniqueCount="3198">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -24578,6 +24578,28 @@
   </si>
   <si>
     <t>Ask for confirmation when deleting sub-entries of triggers/scripts, etc.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>BatchConnectOff</t>
+  </si>
+  <si>
+    <t>BatchConnectOn</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>BatchConnect: On, press 'A' to switch</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>BatchConnect: Off, press 'A' to switch</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>批量连接：开，按A键切换</t>
+  </si>
+  <si>
+    <t>批量连接：关，按A键切换</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -24996,7 +25018,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1120"/>
+  <dimension ref="A1:D1122"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -37318,6 +37340,28 @@
         <v>3190</v>
       </c>
     </row>
+    <row r="1121" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1121" s="3" t="s">
+        <v>3193</v>
+      </c>
+      <c r="B1121" s="4" t="s">
+        <v>3196</v>
+      </c>
+      <c r="C1121" s="3" t="s">
+        <v>3194</v>
+      </c>
+    </row>
+    <row r="1122" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1122" s="3" t="s">
+        <v>3192</v>
+      </c>
+      <c r="B1122" s="4" t="s">
+        <v>3197</v>
+      </c>
+      <c r="C1122" s="3" t="s">
+        <v>3195</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
improve path distance tool
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4A23FD4-2FBF-4A21-8DAC-E1585B94044A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C03CA23D-C1C8-4BC1-AA3E-BEC972BC03EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3020" yWindow="760" windowWidth="28900" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3360" uniqueCount="3198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3369" uniqueCount="3203">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -24385,13 +24385,6 @@
     <t>寻路测距</t>
   </si>
   <si>
-    <t>寻路类型:</t>
-  </si>
-  <si>
-    <t>MeasurementToolbox.MovementZone</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>MeasurementToolbox.PathDistanceGroup</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -24400,21 +24393,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>MeasurementToolbox.DestructibleOverlay</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>MeasurementToolbox.DestructibleUnits</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>可摧毁\n单位</t>
-  </si>
-  <si>
-    <t>可摧毁\n覆盖物</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>MeasurementToolbox.ClearPathDistance</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -24457,15 +24435,6 @@
     <t>Path Distance</t>
   </si>
   <si>
-    <t>MovementZone:</t>
-  </si>
-  <si>
-    <t>Destructible\nOverlay</t>
-  </si>
-  <si>
-    <t>Destructible\nUnits</t>
-  </si>
-  <si>
     <t>Clear Paths</t>
   </si>
   <si>
@@ -24600,6 +24569,56 @@
   </si>
   <si>
     <t>批量连接：关，按A键切换</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MeasurementToolbox.SubjectToText</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>受阻碍：</t>
+  </si>
+  <si>
+    <t>覆盖物</t>
+  </si>
+  <si>
+    <t>MeasurementToolbox.SubjectToBuilding</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MeasurementToolbox.SubjectToTree</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>树木</t>
+  </si>
+  <si>
+    <t>Subject to:</t>
+  </si>
+  <si>
+    <t>Overlay</t>
+  </si>
+  <si>
+    <t>Tree</t>
+  </si>
+  <si>
+    <t>MeasurementToolbox.SubjectToOverlay</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MeasurementToolbox.PathObjectType.Vehicle</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>MeasurementToolbox.PathObjectType.Infantry</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>车辆</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>步兵</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -25018,7 +25037,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1122"/>
+  <dimension ref="A1:D1125"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -37111,255 +37130,288 @@
     </row>
     <row r="1100" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1100" s="3" t="s">
-        <v>3135</v>
+        <v>3133</v>
       </c>
       <c r="B1100" s="4" t="s">
         <v>3130</v>
       </c>
       <c r="C1100" s="3" t="s">
-        <v>3150</v>
+        <v>3144</v>
       </c>
     </row>
     <row r="1101" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1101" s="3" t="s">
-        <v>3134</v>
+        <v>3132</v>
       </c>
       <c r="B1101" s="4" t="s">
         <v>3131</v>
       </c>
       <c r="C1101" s="3" t="s">
-        <v>3150</v>
-      </c>
-    </row>
-    <row r="1102" spans="1:3" x14ac:dyDescent="0.4">
+        <v>3144</v>
+      </c>
+    </row>
+    <row r="1102" spans="1:3" ht="38" x14ac:dyDescent="0.4">
       <c r="A1102" s="3" t="s">
-        <v>3133</v>
+        <v>3199</v>
       </c>
       <c r="B1102" s="4" t="s">
-        <v>3132</v>
+        <v>3201</v>
       </c>
       <c r="C1102" s="3" t="s">
-        <v>3151</v>
-      </c>
-    </row>
-    <row r="1103" spans="1:3" x14ac:dyDescent="0.4">
+        <v>1010</v>
+      </c>
+    </row>
+    <row r="1103" spans="1:3" ht="38" x14ac:dyDescent="0.4">
       <c r="A1103" s="3" t="s">
-        <v>3136</v>
+        <v>3200</v>
       </c>
       <c r="B1103" s="4" t="s">
-        <v>3139</v>
+        <v>3202</v>
       </c>
       <c r="C1103" s="3" t="s">
-        <v>3152</v>
+        <v>1009</v>
       </c>
     </row>
     <row r="1104" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1104" s="3" t="s">
-        <v>3137</v>
+        <v>3189</v>
       </c>
       <c r="B1104" s="4" t="s">
-        <v>3138</v>
+        <v>3190</v>
       </c>
       <c r="C1104" s="3" t="s">
-        <v>3153</v>
+        <v>3195</v>
       </c>
     </row>
     <row r="1105" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1105" s="3" t="s">
+        <v>3198</v>
+      </c>
+      <c r="B1105" s="4" t="s">
+        <v>3191</v>
+      </c>
+      <c r="C1105" s="3" t="s">
+        <v>3196</v>
+      </c>
+    </row>
+    <row r="1106" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1106" s="3" t="s">
+        <v>3192</v>
+      </c>
+      <c r="B1106" s="4" t="s">
+        <v>3057</v>
+      </c>
+      <c r="C1106" s="3" t="s">
+        <v>903</v>
+      </c>
+    </row>
+    <row r="1107" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1107" s="3" t="s">
+        <v>3193</v>
+      </c>
+      <c r="B1107" s="4" t="s">
+        <v>3194</v>
+      </c>
+      <c r="C1107" s="3" t="s">
+        <v>3197</v>
+      </c>
+    </row>
+    <row r="1108" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1108" s="3" t="s">
+        <v>3134</v>
+      </c>
+      <c r="B1108" s="4" t="s">
+        <v>3135</v>
+      </c>
+      <c r="C1108" s="3" t="s">
+        <v>3145</v>
+      </c>
+    </row>
+    <row r="1109" spans="1:3" ht="38" x14ac:dyDescent="0.4">
+      <c r="A1109" s="3" t="s">
+        <v>3136</v>
+      </c>
+      <c r="B1109" s="4" t="s">
+        <v>3139</v>
+      </c>
+      <c r="C1109" s="3" t="s">
+        <v>3146</v>
+      </c>
+    </row>
+    <row r="1110" spans="1:3" ht="38" x14ac:dyDescent="0.4">
+      <c r="A1110" s="3" t="s">
+        <v>3137</v>
+      </c>
+      <c r="B1110" s="4" t="s">
         <v>3140</v>
       </c>
-      <c r="B1105" s="4" t="s">
+      <c r="C1110" s="3" t="s">
+        <v>3147</v>
+      </c>
+    </row>
+    <row r="1111" spans="1:3" ht="38" x14ac:dyDescent="0.4">
+      <c r="A1111" s="3" t="s">
+        <v>3138</v>
+      </c>
+      <c r="B1111" s="4" t="s">
         <v>3141</v>
       </c>
-      <c r="C1105" s="3" t="s">
-        <v>3154</v>
-      </c>
-    </row>
-    <row r="1106" spans="1:3" ht="38" x14ac:dyDescent="0.4">
-      <c r="A1106" s="3" t="s">
+      <c r="C1111" s="3" t="s">
+        <v>3148</v>
+      </c>
+    </row>
+    <row r="1112" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1112" s="3" t="s">
+        <v>3143</v>
+      </c>
+      <c r="B1112" s="4" t="s">
         <v>3142</v>
       </c>
-      <c r="B1106" s="4" t="s">
-        <v>3145</v>
-      </c>
-      <c r="C1106" s="3" t="s">
-        <v>3155</v>
-      </c>
-    </row>
-    <row r="1107" spans="1:3" ht="38" x14ac:dyDescent="0.4">
-      <c r="A1107" s="3" t="s">
-        <v>3143</v>
-      </c>
-      <c r="B1107" s="4" t="s">
-        <v>3146</v>
-      </c>
-      <c r="C1107" s="3" t="s">
-        <v>3156</v>
-      </c>
-    </row>
-    <row r="1108" spans="1:3" ht="38" x14ac:dyDescent="0.4">
-      <c r="A1108" s="3" t="s">
-        <v>3144</v>
-      </c>
-      <c r="B1108" s="4" t="s">
-        <v>3147</v>
-      </c>
-      <c r="C1108" s="3" t="s">
-        <v>3157</v>
-      </c>
-    </row>
-    <row r="1109" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A1109" s="3" t="s">
+      <c r="C1112" s="3" t="s">
         <v>3149</v>
-      </c>
-      <c r="B1109" s="4" t="s">
-        <v>3148</v>
-      </c>
-      <c r="C1109" s="3" t="s">
-        <v>3158</v>
-      </c>
-    </row>
-    <row r="1110" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A1110" s="3" t="s">
-        <v>3159</v>
-      </c>
-      <c r="B1110" s="4" t="s">
-        <v>3161</v>
-      </c>
-      <c r="C1110" s="3" t="s">
-        <v>3163</v>
-      </c>
-    </row>
-    <row r="1111" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A1111" s="3" t="s">
-        <v>3160</v>
-      </c>
-      <c r="B1111" s="4" t="s">
-        <v>3162</v>
-      </c>
-      <c r="C1111" s="3" t="s">
-        <v>3164</v>
-      </c>
-    </row>
-    <row r="1112" spans="1:3" ht="38" x14ac:dyDescent="0.4">
-      <c r="A1112" s="3" t="s">
-        <v>3165</v>
-      </c>
-      <c r="B1112" s="4" t="s">
-        <v>3166</v>
-      </c>
-      <c r="C1112" s="3" t="s">
-        <v>3191</v>
       </c>
     </row>
     <row r="1113" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1113" s="3" t="s">
-        <v>3167</v>
+        <v>3150</v>
       </c>
       <c r="B1113" s="4" t="s">
-        <v>3168</v>
+        <v>3152</v>
       </c>
       <c r="C1113" s="3" t="s">
-        <v>3183</v>
+        <v>3154</v>
       </c>
     </row>
     <row r="1114" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1114" s="3" t="s">
-        <v>3169</v>
+        <v>3151</v>
       </c>
       <c r="B1114" s="4" t="s">
-        <v>3170</v>
+        <v>3153</v>
       </c>
       <c r="C1114" s="3" t="s">
-        <v>3184</v>
-      </c>
-    </row>
-    <row r="1115" spans="1:3" x14ac:dyDescent="0.4">
+        <v>3155</v>
+      </c>
+    </row>
+    <row r="1115" spans="1:3" ht="38" x14ac:dyDescent="0.4">
       <c r="A1115" s="3" t="s">
-        <v>3171</v>
+        <v>3156</v>
       </c>
       <c r="B1115" s="4" t="s">
-        <v>3172</v>
+        <v>3157</v>
       </c>
       <c r="C1115" s="3" t="s">
-        <v>3185</v>
+        <v>3182</v>
       </c>
     </row>
     <row r="1116" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1116" s="3" t="s">
-        <v>3173</v>
+        <v>3158</v>
       </c>
       <c r="B1116" s="4" t="s">
+        <v>3159</v>
+      </c>
+      <c r="C1116" s="3" t="s">
         <v>3174</v>
-      </c>
-      <c r="C1116" s="3" t="s">
-        <v>3186</v>
       </c>
     </row>
     <row r="1117" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1117" s="3" t="s">
+        <v>3160</v>
+      </c>
+      <c r="B1117" s="4" t="s">
+        <v>3161</v>
+      </c>
+      <c r="C1117" s="3" t="s">
         <v>3175</v>
-      </c>
-      <c r="B1117" s="4" t="s">
-        <v>3176</v>
-      </c>
-      <c r="C1117" s="3" t="s">
-        <v>3187</v>
       </c>
     </row>
     <row r="1118" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1118" s="3" t="s">
-        <v>3177</v>
+        <v>3162</v>
       </c>
       <c r="B1118" s="4" t="s">
-        <v>3178</v>
+        <v>3163</v>
       </c>
       <c r="C1118" s="3" t="s">
-        <v>3188</v>
+        <v>3176</v>
       </c>
     </row>
     <row r="1119" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1119" s="3" t="s">
-        <v>3179</v>
+        <v>3164</v>
       </c>
       <c r="B1119" s="4" t="s">
-        <v>3180</v>
+        <v>3165</v>
       </c>
       <c r="C1119" s="3" t="s">
-        <v>3189</v>
+        <v>3177</v>
       </c>
     </row>
     <row r="1120" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1120" s="3" t="s">
-        <v>3181</v>
+        <v>3166</v>
       </c>
       <c r="B1120" s="4" t="s">
-        <v>3182</v>
+        <v>3167</v>
       </c>
       <c r="C1120" s="3" t="s">
-        <v>3190</v>
+        <v>3178</v>
       </c>
     </row>
     <row r="1121" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1121" s="3" t="s">
-        <v>3193</v>
+        <v>3168</v>
       </c>
       <c r="B1121" s="4" t="s">
-        <v>3196</v>
+        <v>3169</v>
       </c>
       <c r="C1121" s="3" t="s">
-        <v>3194</v>
+        <v>3179</v>
       </c>
     </row>
     <row r="1122" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1122" s="3" t="s">
-        <v>3192</v>
+        <v>3170</v>
       </c>
       <c r="B1122" s="4" t="s">
-        <v>3197</v>
+        <v>3171</v>
       </c>
       <c r="C1122" s="3" t="s">
-        <v>3195</v>
+        <v>3180</v>
+      </c>
+    </row>
+    <row r="1123" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1123" s="3" t="s">
+        <v>3172</v>
+      </c>
+      <c r="B1123" s="4" t="s">
+        <v>3173</v>
+      </c>
+      <c r="C1123" s="3" t="s">
+        <v>3181</v>
+      </c>
+    </row>
+    <row r="1124" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1124" s="3" t="s">
+        <v>3184</v>
+      </c>
+      <c r="B1124" s="4" t="s">
+        <v>3187</v>
+      </c>
+      <c r="C1124" s="3" t="s">
+        <v>3185</v>
+      </c>
+    </row>
+    <row r="1125" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1125" s="3" t="s">
+        <v>3183</v>
+      </c>
+      <c r="B1125" s="4" t="s">
+        <v>3188</v>
+      </c>
+      <c r="C1125" s="3" t="s">
+        <v>3186</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
script editor supports jump to waypoint
</commit_message>
<xml_diff>
--- a/Supplementary/文档/FALanguage新增标签.xlsx
+++ b/Supplementary/文档/FALanguage新增标签.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\YURI\源码\FA2spHDM\Supplementary\文档\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C03CA23D-C1C8-4BC1-AA3E-BEC972BC03EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39F51288-93EF-4103-B3F0-319E99CB1B19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3020" yWindow="760" windowWidth="28900" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8820" yWindow="2030" windowWidth="28900" windowHeight="17710" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3369" uniqueCount="3203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3372" uniqueCount="3206">
   <si>
     <t>INIEditorTitle</t>
   </si>
@@ -24620,6 +24620,16 @@
   <si>
     <t>步兵</t>
     <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Options.TileSetBrowserMultiLineTabs</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>地形浏览器标签页多行显示</t>
+  </si>
+  <si>
+    <t>Display tile browser tabs in multiple rows</t>
   </si>
 </sst>
 </file>
@@ -25037,7 +25047,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D1125"/>
+  <dimension ref="A1:D1126"/>
   <sheetFormatPr defaultRowHeight="19.5" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="44.25" style="3" customWidth="1"/>
@@ -37414,6 +37424,17 @@
         <v>3186</v>
       </c>
     </row>
+    <row r="1126" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A1126" s="3" t="s">
+        <v>3203</v>
+      </c>
+      <c r="B1126" s="4" t="s">
+        <v>3204</v>
+      </c>
+      <c r="C1126" s="3" t="s">
+        <v>3205</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>